<commit_message>
feat(mobile): add landscape fullscreen video player
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D410" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A2:D401"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D423" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D415"/>
+  <dimension ref="A1:D423"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8735,6 +8735,182 @@
         <v/>
       </c>
     </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>PLAYER_ENTER_FULLSCREEN</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Enter fullscreen</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Entrar en pantalla completa</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Passer en plein écran</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>PLAYER_EXIT_FULLSCREEN</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Exit fullscreen</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Salir de pantalla completa</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Quitter le plein écran</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>PLAYER_SHOW_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Show video controls</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Mostrar controles de vídeo</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Afficher les commandes vidéo</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>PLAYER_SEEK</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Seek playback position</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Cambiar posición de reproducción</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Changer la position de lecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>PLAYER_REWIND_TEN_SECONDS</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Rewind 10 seconds</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Retroceder 10 segundos</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Reculer de 10 secondes</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>PLAYER_FORWARD_TEN_SECONDS</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Forward 10 seconds</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Avanzar 10 segundos</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Avancer de 10 secondes</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>PLAYER_CLOSE_BOOKMARKS</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Close bookmarks</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Cerrar marcadores</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Fermer les favoris</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>PLAYER_FULLSCREEN_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Fullscreen landscape video is unavailable on this device</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>El vídeo en pantalla completa horizontal no está disponible en este dispositivo</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>La vidéo en plein écran paysage est indisponible sur cet appareil</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Adopt app-template structure and S3-backed storage workflows
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D423"/>
+  <dimension ref="A1:D443"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8911,6 +8911,446 @@
         </is>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_EMPTY</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>No notifications</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>No hay notificaciones</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>No notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_MORE</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Load more</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Cargar más</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Load more</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_LOAD_FAILED</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Could not load notifications</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>No se pudieron cargar las notificaciones</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Could not load notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Notification</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Notificación</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_EVENT_APPLICATION_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Application messages</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Mensajes de la aplicación</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Application messages</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_APPLICATION_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>{MESSAGE}</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>{MESSAGE}</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>{MESSAGE}</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_EVENT_DOWNLOAD_COMPLETED</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Completed downloads</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Descargas completadas</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Completed downloads</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_DOWNLOAD_COMPLETED</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Download completed: {TITLE}</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Descarga completada: {TITLE}</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Download completed: {TITLE}</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_EVENT_DOWNLOAD_FAILED</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Failed downloads</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Descargas fallidas</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Failed downloads</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_DOWNLOAD_FAILED</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Download failed: {TITLE}</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Descarga fallida: {TITLE}</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Download failed: {TITLE}</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_EVENT_BUILD_PUBLISHED</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>New app versions</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Nuevas versiones de la aplicación</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>New app versions</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_BUILD_PUBLISHED</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Version {VERSION} is available</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>La versión {VERSION} está disponible</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Version {VERSION} is available</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_SUBSCRIPTIONS</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Notification subscriptions</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Suscripciones a notificaciones</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Notification subscriptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_SAVE</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Save subscriptions</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Guardar suscripciones</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Save subscriptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_SAVED</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Subscriptions saved</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Suscripciones guardadas</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Subscriptions saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_SELECT_USER</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Select a user</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Selecciona un usuario</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Select a user</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>SETTINGS_SHARE_SHEET_LOGS</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Share logs</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Compartir registros</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Partager les journaux</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>PROFILE_IMAGE</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Profile image</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Imagen de perfil</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Photo de profil</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>PROFILE_IMAGE_CHANGE</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Change profile image</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Cambiar imagen de perfil</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Changer la photo de profil</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(recommendations): settings UI, provider attribution and docs
- Web Settings > Recommendations: opt-in toggle, ListenBrainz username,
  list of providers configured on the server.
- Discover row shows which provider produced it and an inline note when
  external suggestions are unavailable (no toasts, so no repeated alerts).
- Regenerated DTOs / BaseHttp with `python3 -m backend models`.
- New vocabulary keys; docs/RECOMMENDATIONS.md, env vars in docs/DOCKER.md,
  routes in CLAUDE.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUAm7WpakXJtPL79AZPXzr
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D421"/>
+  <dimension ref="A1:D431"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8454,6 +8454,7 @@
         <v/>
       </c>
     </row>
+    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -8851,6 +8852,206 @@
       </c>
       <c r="D421">
         <f>_xlfn.TRANSLATE($B421,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>RECOMMENDATIONS</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="C422">
+        <f>_xlfn.TRANSLATE($B422,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D422">
+        <f>_xlfn.TRANSLATE($B422,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>RECOMMENDATIONS_EXTERNAL_ENABLE</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Use external services for discovery suggestions</t>
+        </is>
+      </c>
+      <c r="C423">
+        <f>_xlfn.TRANSLATE($B423,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D423">
+        <f>_xlfn.TRANSLATE($B423,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>RECOMMENDATIONS_EXTERNAL_HELP</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Local recommendations always work offline and need no setup. When this is on, Rockit may ask ListenBrainz for your recommendations (only your ListenBrainz username is sent) or Last.fm for tracks similar to a song (only that song's artist and title are sent).</t>
+        </is>
+      </c>
+      <c r="C424">
+        <f>_xlfn.TRANSLATE($B424,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D424">
+        <f>_xlfn.TRANSLATE($B424,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>LISTENBRAINZ_USERNAME</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>ListenBrainz username</t>
+        </is>
+      </c>
+      <c r="C425">
+        <f>_xlfn.TRANSLATE($B425,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D425">
+        <f>_xlfn.TRANSLATE($B425,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>LISTENBRAINZ_USERNAME_HELP</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Your public ListenBrainz username, no token needed. ListenBrainz builds recommendations from the listens you submit to it, so new accounts may not get any for a while.</t>
+        </is>
+      </c>
+      <c r="C426">
+        <f>_xlfn.TRANSLATE($B426,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D426">
+        <f>_xlfn.TRANSLATE($B426,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>RECOMMENDATIONS_AVAILABLE_PROVIDERS</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Available on this server</t>
+        </is>
+      </c>
+      <c r="C427">
+        <f>_xlfn.TRANSLATE($B427,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D427">
+        <f>_xlfn.TRANSLATE($B427,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>RECOMMENDATIONS_NO_PROVIDERS</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>No external provider is configured on this server.</t>
+        </is>
+      </c>
+      <c r="C428">
+        <f>_xlfn.TRANSLATE($B428,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D428">
+        <f>_xlfn.TRANSLATE($B428,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>RECOMMENDATIONS_SETTINGS_SAVED</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Recommendation settings saved</t>
+        </is>
+      </c>
+      <c r="C429">
+        <f>_xlfn.TRANSLATE($B429,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D429">
+        <f>_xlfn.TRANSLATE($B429,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>ERROR_SAVING_RECOMMENDATION_SETTINGS</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Could not save recommendation settings</t>
+        </is>
+      </c>
+      <c r="C430">
+        <f>_xlfn.TRANSLATE($B430,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D430">
+        <f>_xlfn.TRANSLATE($B430,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>DISCOVER_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>External suggestions are unavailable right now. Showing local picks.</t>
+        </is>
+      </c>
+      <c r="C431">
+        <f>_xlfn.TRANSLATE($B431,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D431">
+        <f>_xlfn.TRANSLATE($B431,$B$2,D$2)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Paginate download history and complete album and playlist group actions
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D423" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D433" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D423"/>
+  <dimension ref="A1:D433"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8454,7 +8454,6 @@
         <v/>
       </c>
     </row>
-    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -8908,6 +8907,226 @@
       <c r="D423" t="inlineStr">
         <is>
           <t>La vidéo en plein écran paysage est indisponible sur cet appareil</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_NEXT_PAGE</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Next page</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Página siguiente</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Next page</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_PREVIOUS_PAGE</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Previous page</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Página anterior</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Previous page</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_SEARCH</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Search downloads by song, album or playlist</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Buscar descargas por canción, álbum o playlist</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Search downloads by song, album or playlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_DELETE_GROUP</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Delete the downloaded files in this group? This does not delete the source album or playlist.</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>¿Borrar los archivos descargados de este grupo? Esto no borra el álbum o la playlist de origen.</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Delete the downloaded files in this group? This does not delete the source album or playlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_SHOW_TRACKS</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Show tracks</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Ver canciones</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Show tracks</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_HIDE_TRACKS</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Hide tracks</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Ocultar canciones</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Hide tracks</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_AUTO_LIBRARY</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Automatically add downloads to my library</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Añadir las descargas automáticamente a mi biblioteca</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Automatically add downloads to my library</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_PAGE</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Página</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>SETTINGS_SHARE_SHEET_LOGS</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Share sheet logs</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Share sheet logs</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Share sheet logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>DOWNLOADER_ACTIVITY</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Activity over the last 14 days</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Actividad de los últimos 14 días</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Activity over the last 14 days</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix notification vocabulary source and publish images only from main
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D433" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D452" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D433"/>
+  <dimension ref="A1:D452"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9130,6 +9130,424 @@
         </is>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_ALL</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Toutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_CLOSE</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Close notifications</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Cerrar notificaciones</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Fermer les notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_DOWNLOAD_DONE</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Download completed</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Descarga completada</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Téléchargement terminé</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_DOWNLOAD_FAILED</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Download failed</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Descarga fallida</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Échec du téléchargement</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_EMPTY</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>No notifications</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>No hay notificaciones</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Aucune notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_EMPTY_DETAIL</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Downloads, imports and release news will appear here.</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Aquí aparecerán tus descargas, importaciones y novedades.</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Vos téléchargements, importations et nouveautés apparaîtront ici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_IMPORT_DONE</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Import completed</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Importación completada</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Importation terminée</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_IMPORT_FAILED</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Import failed</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Importación fallida</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Échec de l’importation</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_MARK_ALL</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Mark all as read</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Marcar todas como leídas</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Tout marquer comme lu</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_NO_READ</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>No read notifications</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>No hay notificaciones leídas</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Aucune notification lue</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_NO_UNREAD</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>No unread notifications</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>No tienes notificaciones sin leer</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Aucune notification non lue</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_READ</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Mark as read</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Marcar como leída</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Marquer comme lue</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_READ_TAB</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Leídas</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Lues</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_RELEASE_DETAIL</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Check your downloads, imports and updates here.</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Consulta aquí tus descargas, importaciones y novedades.</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Consultez vos téléchargements, importations et nouveautés ici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_RELEASE_TITLE</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Notification center</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Centro de notificaciones</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Centre de notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_TITLE</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Notificaciones</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_UNREAD</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Unread</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Sin leer</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Non lues</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_ZIP_DETAIL</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Save the file from your browser.</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Guarda el archivo desde tu navegador.</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Enregistrez le fichier depuis votre navigateur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>NOTIFICATIONS_ZIP_READY</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>ZIP ready</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>ZIP preparado</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>ZIP prêt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Redesign Friends as an interactive music identity and social league
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D510"/>
+  <dimension ref="A1:D531"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -10739,6 +10739,468 @@
         </is>
       </c>
     </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>SOCIAL_HEADLINE</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Your music. Your people.</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Tu música. Tu gente.</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Votre musique. Vos proches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>SOCIAL_INTRO</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Listen, climb, discover together.</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Escucha, sube de nivel y descubre en compañía.</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Écoutez, progressez, découvrez ensemble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>SOCIAL_PASSPORT</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Your music identity</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Tu identidad musical</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Votre identité musicale</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>SOCIAL_LEVEL</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Level {level}</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Nivel {level}</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Niveau {level}</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>SOCIAL_LISTENS</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Recorded listens</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Escuchas registradas</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Écoutes enregistrées</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>SOCIAL_STREAK</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Day streak</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Días de racha</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Jours consécutifs</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>SOCIAL_NEXT</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>{xp} XP to the next level</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>{xp} XP para el siguiente nivel</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>{xp} XP avant le prochain niveau</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>SOCIAL_MAX</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Highest level reached</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Has alcanzado el nivel máximo</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Niveau maximum atteint</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>SOCIAL_XP_RULE</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>10 XP per recorded listen. All-time stats.</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>10 XP por escucha registrada. Estadísticas acumuladas.</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>10 XP par écoute enregistrée. Statistiques cumulées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>SOCIAL_RACE</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>The listening league</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>La liga de escuchas</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>La ligue des écoutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>SOCIAL_COMPARE</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Choose a friend to compare</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Elige un amigo para compararos</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Choisissez un ami pour comparer</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>SOCIAL_YOU</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Vous</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>SOCIAL_GAP</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>{xp} XP to match {name}</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>{xp} XP para alcanzar a {name}</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>{xp} XP pour rejoindre {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>SOCIAL_LEAD</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>You set the pace. Keep listening.</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Tú marcas el ritmo. Sigue escuchando.</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Vous donnez le rythme. Continuez à écouter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>SOCIAL_TIED</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Same XP. Share your next discovery.</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Mismos XP. Compartid vuestro próximo descubrimiento.</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Même XP. Partagez votre prochaine découverte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>SOCIAL_PEOPLE</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Your circle</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Tu círculo</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Votre cercle</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>SOCIAL_DISCOVER</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>On their headphones</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>En sus auriculares</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Dans leurs écouteurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>SOCIAL_MANAGE</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Find and manage friends</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Buscar y gestionar amigos</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Trouver et gérer des amis</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>SOCIAL_ERROR</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Could not load your league.</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>No se ha podido cargar tu liga.</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Impossible de charger votre ligue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>SOCIAL_RETRY</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Try again</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Reintentar</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Réessayer</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>SOCIAL_EMPTY</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Every league starts with a friend. Invite yours below.</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Toda liga empieza con un amigo. Añade al tuyo aquí abajo.</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Chaque ligue commence avec un ami. Ajoutez le vôtre ci-dessous.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Correct RockIt! branding and complete Friends translations in all languages
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D559"/>
+  <dimension ref="A1:D568"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -704,13 +704,15 @@
           <t>Add to queue</t>
         </is>
       </c>
-      <c r="C13">
-        <f>_xlfn.TRANSLATE(B13,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D13">
-        <f>_xlfn.TRANSLATE(B13,$B$2,D$2)</f>
-        <v/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Añadir a la cola</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ajouter à la file</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2524,13 +2526,15 @@
           <t>Cancel</t>
         </is>
       </c>
-      <c r="C104">
-        <f>_xlfn.TRANSLATE(B104,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D104">
-        <f>_xlfn.TRANSLATE(B104,$B$2,D$2)</f>
-        <v/>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Cancelar</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Annuler</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -2824,13 +2828,15 @@
           <t>Delete</t>
         </is>
       </c>
-      <c r="C119">
-        <f>_xlfn.TRANSLATE(B119,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D119">
-        <f>_xlfn.TRANSLATE(B119,$B$2,D$2)</f>
-        <v/>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Eliminar</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Supprimer</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -4184,13 +4190,15 @@
           <t>Friends</t>
         </is>
       </c>
-      <c r="C187">
-        <f>_xlfn.TRANSLATE(B187,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D187">
-        <f>_xlfn.TRANSLATE(B187,$B$2,D$2)</f>
-        <v/>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Amigos</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Amis</t>
+        </is>
       </c>
     </row>
     <row r="188">
@@ -4204,13 +4212,15 @@
           <t>Friends List</t>
         </is>
       </c>
-      <c r="C188">
-        <f>_xlfn.TRANSLATE(B188,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D188">
-        <f>_xlfn.TRANSLATE(B188,$B$2,D$2)</f>
-        <v/>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Lista de amigos</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Liste d’amis</t>
+        </is>
       </c>
     </row>
     <row r="189">
@@ -4221,16 +4231,18 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Earn points by listening to music, sharing songs, enjoying music with friends, or adding new friends. Keep going and level up!</t>
-        </is>
-      </c>
-      <c r="C189">
-        <f>_xlfn.TRANSLATE(B189,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D189">
-        <f>_xlfn.TRANSLATE(B189,$B$2,D$2)</f>
-        <v/>
+          <t>Earn 10 XP per recorded listen and level up.</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Gana 10 XP por escucha registrada y sube de nivel.</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Gagnez 10 XP par écoute enregistrée et progressez.</t>
+        </is>
       </c>
     </row>
     <row r="190">
@@ -4244,13 +4256,15 @@
           <t>Friends stats</t>
         </is>
       </c>
-      <c r="C190">
-        <f>_xlfn.TRANSLATE(B190,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D190">
-        <f>_xlfn.TRANSLATE(B190,$B$2,D$2)</f>
-        <v/>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Estadísticas de amigos</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Statistiques des amis</t>
+        </is>
       </c>
     </row>
     <row r="191">
@@ -4804,13 +4818,15 @@
           <t>Like</t>
         </is>
       </c>
-      <c r="C218">
-        <f>_xlfn.TRANSLATE(B218,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D218">
-        <f>_xlfn.TRANSLATE(B218,$B$2,D$2)</f>
-        <v/>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Me gusta</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>J’aime</t>
+        </is>
       </c>
     </row>
     <row r="219">
@@ -5924,13 +5940,15 @@
           <t>Pause</t>
         </is>
       </c>
-      <c r="C274">
-        <f>_xlfn.TRANSLATE(B274,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D274">
-        <f>_xlfn.TRANSLATE(B274,$B$2,D$2)</f>
-        <v/>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Pausar</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Mettre en pause</t>
+        </is>
       </c>
     </row>
     <row r="275">
@@ -6144,13 +6162,15 @@
           <t>Play</t>
         </is>
       </c>
-      <c r="C285">
-        <f>_xlfn.TRANSLATE(B285,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D285">
-        <f>_xlfn.TRANSLATE(B285,$B$2,D$2)</f>
-        <v/>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Reproducir</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Lire</t>
+        </is>
       </c>
     </row>
     <row r="286">
@@ -7165,13 +7185,15 @@
           <t>Share song</t>
         </is>
       </c>
-      <c r="C336">
-        <f>_xlfn.TRANSLATE(B336,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D336">
-        <f>_xlfn.TRANSLATE(B336,$B$2,D$2)</f>
-        <v/>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Compartir canción</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Partager le morceau</t>
+        </is>
       </c>
     </row>
     <row r="337">
@@ -7185,13 +7207,15 @@
           <t>Shared Songs for You</t>
         </is>
       </c>
-      <c r="C337">
-        <f>_xlfn.TRANSLATE(B337,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D337">
-        <f>_xlfn.TRANSLATE(B337,$B$2,D$2)</f>
-        <v/>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Canciones compartidas contigo</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Morceaux partagés avec vous</t>
+        </is>
       </c>
     </row>
     <row r="338">
@@ -7205,13 +7229,15 @@
           <t>Shared from</t>
         </is>
       </c>
-      <c r="C338">
-        <f>_xlfn.TRANSLATE(B338,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D338">
-        <f>_xlfn.TRANSLATE(B338,$B$2,D$2)</f>
-        <v/>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Compartido por</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Partagé par</t>
+        </is>
       </c>
     </row>
     <row r="339">
@@ -8454,7 +8480,6 @@
         <v/>
       </c>
     </row>
-    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -9560,13 +9585,15 @@
           <t>Just now</t>
         </is>
       </c>
-      <c r="C453">
-        <f>_xlfn.TRANSLATE($B334,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D453">
-        <f>_xlfn.TRANSLATE($B334,$B$2,D$2)</f>
-        <v/>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Ahora mismo</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>À l’instant</t>
+        </is>
       </c>
     </row>
     <row r="454">
@@ -9580,13 +9607,15 @@
           <t>Nothing playing yet</t>
         </is>
       </c>
-      <c r="C454">
-        <f>_xlfn.TRANSLATE($B335,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D454">
-        <f>_xlfn.TRANSLATE($B335,$B$2,D$2)</f>
-        <v/>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Todavía no suena nada</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Aucune lecture pour le moment</t>
+        </is>
       </c>
     </row>
     <row r="455">
@@ -9600,13 +9629,15 @@
           <t>Your friends' activity will appear here</t>
         </is>
       </c>
-      <c r="C455">
-        <f>_xlfn.TRANSLATE($B336,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D455">
-        <f>_xlfn.TRANSLATE($B336,$B$2,D$2)</f>
-        <v/>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Aquí aparecerá la actividad de tus amigos</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>L’activité de vos amis apparaîtra ici</t>
+        </is>
       </c>
     </row>
     <row r="456">
@@ -9620,13 +9651,15 @@
           <t>Now Playing</t>
         </is>
       </c>
-      <c r="C456">
-        <f>_xlfn.TRANSLATE($B337,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D456">
-        <f>_xlfn.TRANSLATE($B337,$B$2,D$2)</f>
-        <v/>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Sonando ahora</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>En cours de lecture</t>
+        </is>
       </c>
     </row>
     <row r="457">
@@ -9640,13 +9673,15 @@
           <t>Recent</t>
         </is>
       </c>
-      <c r="C457">
-        <f>_xlfn.TRANSLATE($B338,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D457">
-        <f>_xlfn.TRANSLATE($B338,$B$2,D$2)</f>
-        <v/>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Reciente</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Récent</t>
+        </is>
       </c>
     </row>
     <row r="458">
@@ -9660,13 +9695,15 @@
           <t>{count} friends listening now</t>
         </is>
       </c>
-      <c r="C458">
-        <f>_xlfn.TRANSLATE($B339,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D458">
-        <f>_xlfn.TRANSLATE($B339,$B$2,D$2)</f>
-        <v/>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>{count} amigos escuchando ahora</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>{count} amis à l’écoute</t>
+        </is>
       </c>
     </row>
     <row r="459">
@@ -9700,13 +9737,15 @@
           <t>Friend Request</t>
         </is>
       </c>
-      <c r="C460">
-        <f>_xlfn.TRANSLATE($B341,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D460">
-        <f>_xlfn.TRANSLATE($B341,$B$2,D$2)</f>
-        <v/>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Solicitud de amistad</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Demande d’amitié</t>
+        </is>
       </c>
     </row>
     <row r="461">
@@ -9720,13 +9759,15 @@
           <t>Friend Requests</t>
         </is>
       </c>
-      <c r="C461">
-        <f>_xlfn.TRANSLATE($B342,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D461">
-        <f>_xlfn.TRANSLATE($B342,$B$2,D$2)</f>
-        <v/>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Solicitudes de amistad</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Demandes d’amitié</t>
+        </is>
       </c>
     </row>
     <row r="462">
@@ -9760,13 +9801,15 @@
           <t>Listening with</t>
         </is>
       </c>
-      <c r="C463">
-        <f>_xlfn.TRANSLATE($B344,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D463">
-        <f>_xlfn.TRANSLATE($B344,$B$2,D$2)</f>
-        <v/>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Escuchando con</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>À l’écoute avec</t>
+        </is>
       </c>
     </row>
     <row r="464">
@@ -9900,13 +9943,15 @@
           <t>Invite a friend to listen together in real time</t>
         </is>
       </c>
-      <c r="C470">
-        <f>_xlfn.TRANSLATE($B351,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D470">
-        <f>_xlfn.TRANSLATE($B351,$B$2,D$2)</f>
-        <v/>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Invita a un amigo a escuchar contigo</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Invitez un ami à écouter avec vous</t>
+        </is>
       </c>
     </row>
     <row r="471">
@@ -10340,13 +10385,15 @@
           <t>Share</t>
         </is>
       </c>
-      <c r="C492">
-        <f>_xlfn.TRANSLATE($B376,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D492">
-        <f>_xlfn.TRANSLATE($B376,$B$2,D$2)</f>
-        <v/>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Compartir</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Partager</t>
+        </is>
       </c>
     </row>
     <row r="493">
@@ -10420,13 +10467,15 @@
           <t>live</t>
         </is>
       </c>
-      <c r="C496">
-        <f>_xlfn.TRANSLATE($B380,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D496">
-        <f>_xlfn.TRANSLATE($B380,$B$2,D$2)</f>
-        <v/>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>en directo</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>en direct</t>
+        </is>
       </c>
     </row>
     <row r="497">
@@ -11812,6 +11861,204 @@
       <c r="D559" t="inlineStr">
         <is>
           <t>Chaque ligue commence avec un ami. Ajoutez le vôtre ci-dessous.</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>FRIENDS_ACCEPT</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Aceptar</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Accepter</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>FRIENDS_DECLINE</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Decline</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Rechazar</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Refuser</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>SOCIAL_XP</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>SOCIAL_XP_TOTAL</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>{xp} XP</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>{xp} XP</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>{xp} XP</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>SOCIAL_MINUTES_AGO</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>{count}m ago</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>hace {count} min</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>il y a {count} min</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>SOCIAL_HOURS_AGO</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>{count}h ago</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>hace {count} h</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>il y a {count} h</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>SOCIAL_DAYS_AGO</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>{count}d ago</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>hace {count} d</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>il y a {count} j</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>FRIENDS_ACTION_ERROR</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Could not complete this action. Please try again.</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>No se ha podido completar la acción. Inténtalo de nuevo.</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Impossible d’effectuer cette action. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>FRIENDS_LOAD_ERROR</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Could not load your friends. Please try again.</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>No se han podido cargar tus amigos. Inténtalo de nuevo.</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Impossible de charger vos amis. Réessayez.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete download menu vocabulary in Spanish and French
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -644,13 +644,15 @@
           <t>Add to library</t>
         </is>
       </c>
-      <c r="C10">
-        <f>_xlfn.TRANSLATE(B10,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D10">
-        <f>_xlfn.TRANSLATE(B10,$B$2,D$2)</f>
-        <v/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Añadir a la biblioteca</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ajouter à la bibliothèque</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -724,13 +726,15 @@
           <t>Added to library</t>
         </is>
       </c>
-      <c r="C14">
-        <f>_xlfn.TRANSLATE(B14,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D14">
-        <f>_xlfn.TRANSLATE(B14,$B$2,D$2)</f>
-        <v/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Añadido a la biblioteca</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ajouté à la bibliothèque</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2824,13 +2828,15 @@
           <t>Delete</t>
         </is>
       </c>
-      <c r="C119">
-        <f>_xlfn.TRANSLATE(B119,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D119">
-        <f>_xlfn.TRANSLATE(B119,$B$2,D$2)</f>
-        <v/>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Borrar</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Supprimer</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -5164,13 +5170,15 @@
           <t>More Options</t>
         </is>
       </c>
-      <c r="C236">
-        <f>_xlfn.TRANSLATE(B236,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D236">
-        <f>_xlfn.TRANSLATE(B236,$B$2,D$2)</f>
-        <v/>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Más opciones</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Plus d’options</t>
+        </is>
       </c>
     </row>
     <row r="237">
@@ -6564,13 +6572,15 @@
           <t>Redownload</t>
         </is>
       </c>
-      <c r="C306">
-        <f>_xlfn.TRANSLATE(B306,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D306">
-        <f>_xlfn.TRANSLATE(B306,$B$2,D$2)</f>
-        <v/>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Volver a descargar</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Télécharger à nouveau</t>
+        </is>
       </c>
     </row>
     <row r="307">
@@ -8454,6 +8464,7 @@
         <v/>
       </c>
     </row>
+    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -8928,7 +8939,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Next page</t>
+          <t>Page suivante</t>
         </is>
       </c>
     </row>
@@ -8950,7 +8961,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Previous page</t>
+          <t>Page précédente</t>
         </is>
       </c>
     </row>
@@ -8994,7 +9005,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Delete the downloaded files in this group? This does not delete the source album or playlist.</t>
+          <t>Supprimer les fichiers téléchargés de ce groupe ? Cela ne supprime pas l’album ni la playlist d’origine.</t>
         </is>
       </c>
     </row>
@@ -9016,7 +9027,7 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Show tracks</t>
+          <t>Afficher les titres</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9049,7 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Hide tracks</t>
+          <t>Masquer les titres</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix radio discovery, touch playback, and saved station controls
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D452" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D582" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D568"/>
+  <dimension ref="A1:D582"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8488,7 +8488,6 @@
         <v/>
       </c>
     </row>
-    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -12068,6 +12067,314 @@
       <c r="D568" t="inlineStr">
         <is>
           <t>Impossible de charger vos amis. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>RADIO_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Discover the world, one station at a time.</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Descubre el mundo, emisora a emisora.</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Découvrez le monde, une station à la fois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>RADIO_EXPLORE</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Explore</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Explorar</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>RADIO_SAVED</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Saved stations</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Emisoras guardadas</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Stations enregistrées</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>RADIO_COUNTRY</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Choose a country</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Elige un país</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Choisir un pays</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>RADIO_GRID</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Grid view</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Vista de tarjetas</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Vue en grille</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>RADIO_LIST</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>List view</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Vista de lista</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Vue en liste</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>RADIO_CLEAR</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Clear filters</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Limpiar filtros</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Effacer les filtres</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>RADIO_LOADING</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Loading stations…</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Cargando emisoras…</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Chargement des stations…</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>RADIO_LOAD_ERROR</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Stations could not be loaded. Try again.</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>No se han podido cargar las emisoras. Inténtalo de nuevo.</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Impossible de charger les stations. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>RADIO_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>This station has no playable stream.</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Esta emisora no tiene una señal disponible.</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Cette station ne propose aucun flux disponible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>RADIO_MAP_HINT</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Select a country to discover its stations. Saved stations with a location appear on the map.</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Selecciona un país para descubrir sus emisoras. Las guardadas con ubicación aparecen en el mapa.</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Sélectionnez un pays pour découvrir ses stations. Les stations enregistrées avec une position apparaissent sur la carte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>RADIO_EMPTY</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Save stations to your library to find them here and on the map.</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Guarda emisoras en tu biblioteca para encontrarlas aquí y en el mapa.</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Enregistrez des stations dans votre bibliothèque pour les retrouver ici et sur la carte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>PLAYER_ENABLE_SHUFFLE</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Enable shuffle</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Activar reproducción aleatoria</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Activer la lecture aléatoire</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>PLAYER_DISABLE_SHUFFLE</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Disable shuffle</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Desactivar reproducción aleatoria</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Désactiver la lecture aléatoire</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve progressive search and preserve provider choices
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D568"/>
+  <dimension ref="A1:D577"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -584,13 +584,15 @@
           <t>Add media to playlist</t>
         </is>
       </c>
-      <c r="C7">
-        <f>_xlfn.TRANSLATE(B7,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D7">
-        <f>_xlfn.TRANSLATE(B7,$B$2,D$2)</f>
-        <v/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Añadir a una playlist</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ajouter à une playlist</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -686,13 +688,15 @@
           <t>Add to playlist and download</t>
         </is>
       </c>
-      <c r="C12">
-        <f>_xlfn.TRANSLATE(B12,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D12">
-        <f>_xlfn.TRANSLATE(B12,$B$2,D$2)</f>
-        <v/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Añadir a una playlist y descargar</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ajouter à une playlist et télécharger</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2210,13 +2214,15 @@
           <t>Albums</t>
         </is>
       </c>
-      <c r="C88">
-        <f>_xlfn.TRANSLATE(B88,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D88">
-        <f>_xlfn.TRANSLATE(B88,$B$2,D$2)</f>
-        <v/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Álbumes</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Albums</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -2390,13 +2396,15 @@
           <t>Artists</t>
         </is>
       </c>
-      <c r="C97">
-        <f>_xlfn.TRANSLATE(B97,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D97">
-        <f>_xlfn.TRANSLATE(B97,$B$2,D$2)</f>
-        <v/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Artistas</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Artistes</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -2712,13 +2720,15 @@
           <t>Cover of {name}</t>
         </is>
       </c>
-      <c r="C113">
-        <f>_xlfn.TRANSLATE(B113,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D113">
-        <f>_xlfn.TRANSLATE(B113,$B$2,D$2)</f>
-        <v/>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Portada de {name}</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Pochette de {name}</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -2954,13 +2964,15 @@
           <t>Download</t>
         </is>
       </c>
-      <c r="C125">
-        <f>_xlfn.TRANSLATE(B125,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D125">
-        <f>_xlfn.TRANSLATE(B125,$B$2,D$2)</f>
-        <v/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Télécharger</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -2974,13 +2986,15 @@
           <t>Download and Add to Library</t>
         </is>
       </c>
-      <c r="C126">
-        <f>_xlfn.TRANSLATE(B126,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D126">
-        <f>_xlfn.TRANSLATE(B126,$B$2,D$2)</f>
-        <v/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Descargar y añadir a la biblioteca</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Télécharger et ajouter à la bibliothèque</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -2994,13 +3008,15 @@
           <t>Download and Play</t>
         </is>
       </c>
-      <c r="C127">
-        <f>_xlfn.TRANSLATE(B127,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D127">
-        <f>_xlfn.TRANSLATE(B127,$B$2,D$2)</f>
-        <v/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Descargar y reproducir</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Télécharger et lire</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -3154,13 +3170,15 @@
           <t>Download started</t>
         </is>
       </c>
-      <c r="C135">
-        <f>_xlfn.TRANSLATE(B135,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D135">
-        <f>_xlfn.TRANSLATE(B135,$B$2,D$2)</f>
-        <v/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Descarga iniciada</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Téléchargement lancé</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -3174,13 +3192,15 @@
           <t>Download to Server</t>
         </is>
       </c>
-      <c r="C136">
-        <f>_xlfn.TRANSLATE(B136,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D136">
-        <f>_xlfn.TRANSLATE(B136,$B$2,D$2)</f>
-        <v/>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Descargar al servidor</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Télécharger sur le serveur</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -3194,13 +3214,15 @@
           <t>Download ZIP</t>
         </is>
       </c>
-      <c r="C137">
-        <f>_xlfn.TRANSLATE(B137,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D137">
-        <f>_xlfn.TRANSLATE(B137,$B$2,D$2)</f>
-        <v/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Descargar ZIP</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Télécharger le ZIP</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -3914,13 +3936,15 @@
           <t>Error searching</t>
         </is>
       </c>
-      <c r="C173">
-        <f>_xlfn.TRANSLATE(B173,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D173">
-        <f>_xlfn.TRANSLATE(B173,$B$2,D$2)</f>
-        <v/>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Error al buscar</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Erreur lors de la recherche</t>
+        </is>
       </c>
     </row>
     <row r="174">
@@ -6310,13 +6334,15 @@
           <t>Playlists</t>
         </is>
       </c>
-      <c r="C292">
-        <f>_xlfn.TRANSLATE(B292,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D292">
-        <f>_xlfn.TRANSLATE(B292,$B$2,D$2)</f>
-        <v/>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Listas de reproducción</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Playlists</t>
+        </is>
       </c>
     </row>
     <row r="293">
@@ -6510,13 +6536,15 @@
           <t>Radio Stations</t>
         </is>
       </c>
-      <c r="C302">
-        <f>_xlfn.TRANSLATE(B302,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D302">
-        <f>_xlfn.TRANSLATE(B302,$B$2,D$2)</f>
-        <v/>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Emisoras de radio</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Stations de radio</t>
+        </is>
       </c>
     </row>
     <row r="303">
@@ -6732,13 +6760,15 @@
           <t>Remove from library</t>
         </is>
       </c>
-      <c r="C313">
-        <f>_xlfn.TRANSLATE(B313,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D313">
-        <f>_xlfn.TRANSLATE(B313,$B$2,D$2)</f>
-        <v/>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Eliminar de la biblioteca</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Retirer de la bibliothèque</t>
+        </is>
       </c>
     </row>
     <row r="314">
@@ -6912,13 +6942,15 @@
           <t>Retry</t>
         </is>
       </c>
-      <c r="C322">
-        <f>_xlfn.TRANSLATE(B322,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D322">
-        <f>_xlfn.TRANSLATE(B322,$B$2,D$2)</f>
-        <v/>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Reintentar</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Réessayer</t>
+        </is>
       </c>
     </row>
     <row r="323">
@@ -7012,13 +7044,15 @@
           <t>Search</t>
         </is>
       </c>
-      <c r="C327">
-        <f>_xlfn.TRANSLATE(B327,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D327">
-        <f>_xlfn.TRANSLATE(B327,$B$2,D$2)</f>
-        <v/>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Buscar</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Rechercher</t>
+        </is>
       </c>
     </row>
     <row r="328">
@@ -7032,13 +7066,15 @@
           <t>Search for artists, songs, albums...</t>
         </is>
       </c>
-      <c r="C328">
-        <f>_xlfn.TRANSLATE(B328,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D328">
-        <f>_xlfn.TRANSLATE(B328,$B$2,D$2)</f>
-        <v/>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Busca artistas, canciones, álbumes…</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Recherchez des artistes, des titres, des albums…</t>
+        </is>
       </c>
     </row>
     <row r="329">
@@ -7052,13 +7088,15 @@
           <t>It seems silence is also music...</t>
         </is>
       </c>
-      <c r="C329">
-        <f>_xlfn.TRANSLATE(B329,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D329">
-        <f>_xlfn.TRANSLATE(B329,$B$2,D$2)</f>
-        <v/>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Parece que el silencio también es música…</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Il paraît que le silence est aussi de la musique…</t>
+        </is>
       </c>
     </row>
     <row r="330">
@@ -7072,13 +7110,15 @@
           <t>But it's not very entertaining, is it? Find something to listen to!</t>
         </is>
       </c>
-      <c r="C330">
-        <f>_xlfn.TRANSLATE(B330,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D330">
-        <f>_xlfn.TRANSLATE(B330,$B$2,D$2)</f>
-        <v/>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</t>
+        </is>
       </c>
     </row>
     <row r="331">
@@ -7319,13 +7359,15 @@
           <t>Songs</t>
         </is>
       </c>
-      <c r="C342">
-        <f>_xlfn.TRANSLATE(B342,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D342">
-        <f>_xlfn.TRANSLATE(B342,$B$2,D$2)</f>
-        <v/>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Canciones</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Titres</t>
+        </is>
       </c>
     </row>
     <row r="343">
@@ -8359,13 +8401,15 @@
           <t>Videos</t>
         </is>
       </c>
-      <c r="C394">
-        <f>_xlfn.TRANSLATE(B394,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D394">
-        <f>_xlfn.TRANSLATE(B394,$B$2,D$2)</f>
-        <v/>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Vídeos</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Vidéos</t>
+        </is>
       </c>
     </row>
     <row r="395">
@@ -12068,6 +12112,204 @@
       <c r="D568" t="inlineStr">
         <is>
           <t>Impossible de charger vos amis. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>SEARCH_LOAD_MORE</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Load more</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Cargar más</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Afficher plus</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>SEARCH_NO_RESULTS</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>No results found. Try another search.</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>No hay resultados. Prueba otra búsqueda.</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Aucun résultat. Essayez une autre recherche.</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>SEARCH_LOADING</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Searching…</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Buscando…</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Recherche en cours…</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>SEARCH_CHOOSE_SOURCE</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Choose a source</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Elige una fuente</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Choisissez une source</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>SEARCH_SOURCE_DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Downloaded</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Descargado</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Téléchargé</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>SEARCH_ADD_TO_LIBRARY_FROM</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Add to library with {provider}</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Añadir a la biblioteca con {provider}</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Ajouter à la bibliothèque avec {provider}</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>SEARCH_DOWNLOAD_FROM</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Download with {provider}</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Descargar con {provider}</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Télécharger avec {provider}</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>SEARCH_DOWNLOAD_AND_ADD_FROM</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Download and add to library with {provider}</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Descargar y añadir a la biblioteca con {provider}</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Télécharger et ajouter à la bibliothèque avec {provider}</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>SEARCH_PLAY_FROM</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Download and play with {provider}</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Descargar y reproducir con {provider}</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Télécharger et lire avec {provider}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(recommendations): enable server-wide Last.fm and retire per-user settings
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D612"/>
+  <dimension ref="A1:D604"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12864,179 +12864,19 @@
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>RECOMMENDATIONS_EXTERNAL_ENABLE</t>
+          <t>DISCOVER_UNAVAILABLE</t>
         </is>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>Use external services for discovery suggestions</t>
+          <t>External suggestions are unavailable right now. Showing local picks.</t>
         </is>
       </c>
       <c r="C604">
-        <f>_xlfn.TRANSLATE($B423,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B431,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D604">
-        <f>_xlfn.TRANSLATE($B423,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="605">
-      <c r="A605" t="inlineStr">
-        <is>
-          <t>RECOMMENDATIONS_EXTERNAL_HELP</t>
-        </is>
-      </c>
-      <c r="B605" t="inlineStr">
-        <is>
-          <t>Local recommendations always work offline and need no setup. When this is on, Rockit may ask ListenBrainz for your recommendations (only your ListenBrainz username is sent) or Last.fm for tracks similar to a song (only that song's artist and title are sent).</t>
-        </is>
-      </c>
-      <c r="C605">
-        <f>_xlfn.TRANSLATE($B424,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D605">
-        <f>_xlfn.TRANSLATE($B424,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="606">
-      <c r="A606" t="inlineStr">
-        <is>
-          <t>LISTENBRAINZ_USERNAME</t>
-        </is>
-      </c>
-      <c r="B606" t="inlineStr">
-        <is>
-          <t>ListenBrainz username</t>
-        </is>
-      </c>
-      <c r="C606">
-        <f>_xlfn.TRANSLATE($B425,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D606">
-        <f>_xlfn.TRANSLATE($B425,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="607">
-      <c r="A607" t="inlineStr">
-        <is>
-          <t>LISTENBRAINZ_USERNAME_HELP</t>
-        </is>
-      </c>
-      <c r="B607" t="inlineStr">
-        <is>
-          <t>Your public ListenBrainz username, no token needed. ListenBrainz builds recommendations from the listens you submit to it, so new accounts may not get any for a while.</t>
-        </is>
-      </c>
-      <c r="C607">
-        <f>_xlfn.TRANSLATE($B426,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D607">
-        <f>_xlfn.TRANSLATE($B426,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="608">
-      <c r="A608" t="inlineStr">
-        <is>
-          <t>RECOMMENDATIONS_AVAILABLE_PROVIDERS</t>
-        </is>
-      </c>
-      <c r="B608" t="inlineStr">
-        <is>
-          <t>Available on this server</t>
-        </is>
-      </c>
-      <c r="C608">
-        <f>_xlfn.TRANSLATE($B427,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D608">
-        <f>_xlfn.TRANSLATE($B427,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="609">
-      <c r="A609" t="inlineStr">
-        <is>
-          <t>RECOMMENDATIONS_NO_PROVIDERS</t>
-        </is>
-      </c>
-      <c r="B609" t="inlineStr">
-        <is>
-          <t>No external provider is configured on this server.</t>
-        </is>
-      </c>
-      <c r="C609">
-        <f>_xlfn.TRANSLATE($B428,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D609">
-        <f>_xlfn.TRANSLATE($B428,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="610">
-      <c r="A610" t="inlineStr">
-        <is>
-          <t>RECOMMENDATIONS_SETTINGS_SAVED</t>
-        </is>
-      </c>
-      <c r="B610" t="inlineStr">
-        <is>
-          <t>Recommendation settings saved</t>
-        </is>
-      </c>
-      <c r="C610">
-        <f>_xlfn.TRANSLATE($B429,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D610">
-        <f>_xlfn.TRANSLATE($B429,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="611">
-      <c r="A611" t="inlineStr">
-        <is>
-          <t>ERROR_SAVING_RECOMMENDATION_SETTINGS</t>
-        </is>
-      </c>
-      <c r="B611" t="inlineStr">
-        <is>
-          <t>Could not save recommendation settings</t>
-        </is>
-      </c>
-      <c r="C611">
-        <f>_xlfn.TRANSLATE($B430,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D611">
-        <f>_xlfn.TRANSLATE($B430,$B$2,D$2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="612">
-      <c r="A612" t="inlineStr">
-        <is>
-          <t>DISCOVER_UNAVAILABLE</t>
-        </is>
-      </c>
-      <c r="B612" t="inlineStr">
-        <is>
-          <t>External suggestions are unavailable right now. Showing local picks.</t>
-        </is>
-      </c>
-      <c r="C612">
-        <f>_xlfn.TRANSLATE($B431,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D612">
         <f>_xlfn.TRANSLATE($B431,$B$2,D$2)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat(artists): add borderless artist collection and discography experience
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D452" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D609" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D591"/>
+  <dimension ref="A1:D609"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12621,6 +12621,402 @@
         </is>
       </c>
     </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>ARTIST_SONGS</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>songs</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>canciones</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>titres</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>ARTIST_ALBUMS</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>albums</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>álbumes</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>albums</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>ARTIST_PLAY</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Play collection</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Reproducir colección</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Écouter la collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>ARTIST_SOURCE</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Open in</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Abrir en</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Ouvrir dans</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>ARTIST_COLLECTION</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Your collection</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Tu colección</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Votre collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>ARTIST_DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Downloaded</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Descargadas</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Téléchargés</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>ARTIST_SEARCH</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Find a song in the loaded collection</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Buscar entre las canciones cargadas</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Rechercher parmi les titres chargés</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>ARTIST_DOWNLOAD</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Télécharger</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>ARTIST_DISCOGRAPHY</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Discography</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Discografía</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Discographie</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>ARTIST_EMPTY</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>No songs indexed for this artist yet.</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Todavía no hay canciones indexadas de este artista.</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Aucun titre indexé pour cet artiste pour le moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>ARTIST_NO_MATCHES</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>No matching songs in the loaded collection.</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>No hay coincidencias entre las canciones cargadas.</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Aucun titre correspondant parmi les titres chargés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>ARTIST_NO_ALBUMS</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>No albums indexed yet.</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Todavía no hay álbumes indexados.</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Aucun album indexé pour le moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>ARTIST_RELATED</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Connected artists</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Artistas vinculados</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Artistes liés</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>ARTIST_PARTIAL</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Some sources are unavailable or contain ambiguous artist names. Their results have been omitted.</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Algunas fuentes no están disponibles o contienen nombres de artista ambiguos. Se han omitido sus resultados.</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Certaines sources sont indisponibles ou contiennent des noms ambigus. Leurs résultats ont été omis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>ARTIST_LOAD_ERROR</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Could not load more music. Try again.</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>No se pudo cargar más música. Vuelve a intentarlo.</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Impossible de charger plus de musique. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>ARTIST_LOADING</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Loading music…</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Cargando música…</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Chargement de la musique…</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>ARTIST_MORE</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Load more music</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Cargar más música</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Charger plus de musique</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>ARTIST_LOCAL_NOTE</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Music indexed by your sources. Playback and search use the songs loaded on this page. Downloads are marked with a check.</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Música indexada por tus fuentes. La reproducción y la búsqueda usan las canciones cargadas en esta página. Las descargas se indican con una marca.</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Musique indexée par vos sources. La lecture et la recherche utilisent les titres chargés sur cette page. Une coche indique les téléchargements.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(artists): connect MusicBrainz catalogs and compact collection previews
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D609" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D623" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D609"/>
+  <dimension ref="A1:D623"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -13017,6 +13017,314 @@
         </is>
       </c>
     </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>ARTIST_LESS</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Show less</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Ver menos</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Voir moins</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>ARTIST_EXPLORE</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Beyond your collection</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Más allá de tu colección</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Au-delà de votre collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_LOADING</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Looking up the artist catalog…</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Consultando el catálogo del artista…</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Recherche du catalogue de l’artiste…</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_ERROR</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Artist information could not be loaded.</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>No se pudo cargar la información del artista.</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Impossible de charger les informations de l’artiste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_RETRY</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Try again</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Volver a intentar</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Réessayer</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_EMPTY</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>No catalog information found.</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>No se encontró información en el catálogo.</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Aucune information trouvée dans le catalogue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_IDENTITY</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Artist in the external catalog</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Artista en el catálogo externo</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Artiste dans le catalogue externe</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_CHOOSE</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Choose the matching artist</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Elige el artista correspondiente</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Choisissez l’artiste correspondant</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_STALE</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Showing saved information; the source is temporarily unavailable.</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Mostrando información guardada; la fuente no está disponible temporalmente.</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Informations enregistrées ; la source est temporairement indisponible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_EVENTS</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Documented events</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Eventos documentados</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Événements documentés</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_NO_EVENTS</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>No events documented here. This is not a complete concert calendar.</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>No hay eventos documentados aquí. No es una agenda completa de conciertos.</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Aucun événement documenté ici. Ce calendrier de concerts n’est pas exhaustif.</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_ALBUMS</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Discography</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Discografía</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Discographie</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_RECORDINGS</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Recordings</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Grabaciones</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Enregistrements</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_NOTE</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>MusicBrainz metadata, including music outside your collection. Links open the source; they do not play or download music. Releases on loaded pages appear newest first. This catalog does not provide popularity rankings.</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Metadatos de MusicBrainz, también de música fuera de tu colección. Los enlaces abren la fuente; no reproducen ni descargan música. Los lanzamientos de las páginas cargadas se ordenan del más reciente al más antiguo. Este catálogo no ofrece rankings de popularidad.</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Métadonnées MusicBrainz, y compris hors de votre collection. Les liens ouvrent la source, sans lecture ni téléchargement. Les parutions des pages chargées sont triées de la plus récente à la plus ancienne. Ce catalogue ne fournit pas de classement de popularité.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
refactor(artists): prioritize collection and discography with compact context
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D623" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D629" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D423"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D623"/>
+  <dimension ref="A1:D629"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12981,17 +12981,17 @@
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>Load more music</t>
+          <t>Show more</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
         <is>
-          <t>Cargar más música</t>
+          <t>Ver más</t>
         </is>
       </c>
       <c r="D608" t="inlineStr">
         <is>
-          <t>Charger plus de musique</t>
+          <t>Voir plus</t>
         </is>
       </c>
     </row>
@@ -13157,17 +13157,17 @@
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>Artist in the external catalog</t>
+          <t>Several artists share this name</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>Artista en el catálogo externo</t>
+          <t>Varios artistas comparten este nombre</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
         <is>
-          <t>Artiste dans le catalogue externe</t>
+          <t>Plusieurs artistes portent ce nom</t>
         </is>
       </c>
     </row>
@@ -13179,17 +13179,17 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>Choose the matching artist</t>
+          <t>Which artist are you looking for?</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>Elige el artista correspondiente</t>
+          <t>¿Qué artista estás buscando?</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Choisissez l’artiste correspondant</t>
+          <t>Quel artiste recherchez-vous ?</t>
         </is>
       </c>
     </row>
@@ -13223,17 +13223,17 @@
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>Documented events</t>
+          <t>Concerts</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>Eventos documentados</t>
+          <t>Conciertos</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Événements documentés</t>
+          <t>Concerts</t>
         </is>
       </c>
     </row>
@@ -13289,17 +13289,17 @@
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>Recordings</t>
+          <t>More songs and versions</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Grabaciones</t>
+          <t>Más canciones y versiones</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>Enregistrements</t>
+          <t>Plus de titres et de versions</t>
         </is>
       </c>
     </row>
@@ -13322,6 +13322,138 @@
       <c r="D623" t="inlineStr">
         <is>
           <t>Métadonnées MusicBrainz, y compris hors de votre collection. Les liens ouvrent la source, sans lecture ni téléchargement. Les parutions des pages chargées sont triées de la plus récente à la plus ancienne. Ce catalogue ne fournit pas de classement de popularité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>ARTIST_KNOWN_CATALOG</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Known catalog · includes undownloaded music and different editions</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Catálogo conocido · incluye música sin descargar y distintas ediciones</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Catalogue connu · inclut la musique non téléchargée et différentes éditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>ARTIST_NO_UPCOMING_EVENTS</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>No upcoming concerts listed.</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>No hay próximos conciertos registrados.</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Aucun concert à venir répertorié.</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>ARTIST_EVENT_HISTORY</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Past concerts</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Conciertos anteriores</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Concerts passés</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>ARTIST_CATALOG_AVAILABLE</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Explore the catalog · releases and editions</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Explora el catálogo · lanzamientos y ediciones</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Explorer le catalogue · parutions et éditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>ARTIST_OPEN_ALBUM</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Open album</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Abrir álbum</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Ouvrir l’album</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>ARTIST_FIND_MUSIC</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Find in Rockit</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Buscar en Rockit</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Rechercher dans Rockit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(artists): download catalog releases in place and simplify artist layout
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D629"/>
+  <dimension ref="A1:D632"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -13457,6 +13457,72 @@
         </is>
       </c>
     </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>ARTIST_RELEASES</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>releases</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>lanzamientos</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>sorties</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>ARTIST_SOURCE_CHOOSER</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Choose a source</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Elige una fuente</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Choisir une source</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>ARTIST_COLLECTION_EMPTY</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>No music saved yet.</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Todavía no hay música guardada.</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Aucune musique enregistrée pour le moment.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(artists): stabilize discography and refine artist context
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D632"/>
+  <dimension ref="A1:D634"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -13289,17 +13289,17 @@
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>More songs and versions</t>
+          <t>Recordings</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Más canciones y versiones</t>
+          <t>Grabaciones</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>Plus de titres et de versions</t>
+          <t>Enregistrements</t>
         </is>
       </c>
     </row>
@@ -13520,6 +13520,50 @@
       <c r="D632" t="inlineStr">
         <is>
           <t>Aucune musique enregistrée pour le moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>ARTIST_DISCOGRAPHY_SEARCH</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Search discography</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Buscar en la discografía</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Rechercher dans la discographie</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>ARTIST_METADATA_OPTIONS</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Artist options</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Opciones del artista</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Options de l’artiste</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(artists): filter discography without automatic catalog crawling
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D634"/>
+  <dimension ref="A1:D644"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -13567,6 +13567,226 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_TYPES</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Release type</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Tipo de lanzamiento</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Type de sortie</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_ALBUM</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Albums</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Álbumes</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Albums</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_SINGLE</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Singles</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Singles</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Singles</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_EP</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>EPs</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_LIVE</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>En directo</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>En concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_COMPILATION</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Compilations</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Recopilatorios</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Compilations</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_REMIX</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Remixes</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Remixes</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Remixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_SOUNDTRACK</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Soundtracks</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Bandas sonoras</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Bandes originales</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_OTHER</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Autres</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>ARTIST_FILTER_LOADED</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Search and filters apply to loaded releases. Load more to include the next page.</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>La búsqueda y los filtros se aplican a los lanzamientos cargados. Carga más para incluir la siguiente página.</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>La recherche et les filtres portent sur les sorties chargées. Chargez la suite pour inclure la page suivante.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(ci): translate search playback labels in vocabulary [KB-25]
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -6012,13 +6012,15 @@
           <t>Pause {name}</t>
         </is>
       </c>
-      <c r="C276">
-        <f>_xlfn.TRANSLATE(B276,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D276">
-        <f>_xlfn.TRANSLATE(B276,$B$2,D$2)</f>
-        <v/>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Pausar {name}</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Mettre en pause {name}</t>
+        </is>
       </c>
     </row>
     <row r="277">
@@ -6294,13 +6296,15 @@
           <t>Play {name}</t>
         </is>
       </c>
-      <c r="C290">
-        <f>_xlfn.TRANSLATE(B290,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D290">
-        <f>_xlfn.TRANSLATE(B290,$B$2,D$2)</f>
-        <v/>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Reproducir {name}</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Lire {name}</t>
+        </is>
       </c>
     </row>
     <row r="291">

</xml_diff>

<commit_message>
fix(i18n): generate Friends labels from vocabulary workbook [KB-34]
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -435,12 +435,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D657"/>
+  <dimension ref="A1:D668"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8532,7 +8532,6 @@
         <v/>
       </c>
     </row>
-    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -14045,12 +14044,254 @@
       <c r="D657">
         <f>_xlfn.TRANSLATE($B657,$B$2,D$2)</f>
         <v/>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>FRIENDS_SOCIAL_INTRO</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Find your people, share your music.</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Tu gente, vuestra música.</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Vos proches, votre musique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARED_MUSIC</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Music shared with you</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Música que te han compartido</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Musique partagée avec vous</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>FRIENDS_RECENT_LISTENS</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Recently in your circle</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Últimas escuchas de tu círculo</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Écoutes récentes de votre cercle</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>FRIENDS_PERSONAL_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Your listening progress</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Tu progreso de escucha</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Votre progression musicale</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>FRIENDS_ONLINE_COUNT</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>{count} online</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>{count} en línea</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>{count} en ligne</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARED_FROM</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>From {name}</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>De {name}</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>De {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARED_TO</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>To {name}</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Para {name}</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Pour {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHOW_ALL</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Show all {count} friends</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Ver los {count} amigos</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Voir les {count} amis</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHOW_LESS</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Show fewer</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Ver menos</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Voir moins</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>FRIENDS_NAV_SHARED</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Compartidos</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Partagés</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>FRIENDS_NAV_RECENT</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Recent</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Recientes</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>Récentes</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(social): award durable XP for listening-time milestones [KB-35]
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D668"/>
+  <dimension ref="A1:D677"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -14288,6 +14288,204 @@
         </is>
       </c>
     </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>FRIENDS_XP_TIME_RULE</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>XP for verified listening time. Previous XP is preserved.</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>XP por tiempo de escucha verificado. Se conserva tu XP anterior.</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>XP pour le temps d’écoute vérifié. Votre XP antérieure est conservée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>FRIENDS_SESSION_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>This listening session</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Esta sesión de escucha</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Cette session d’écoute</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>FRIENDS_SESSION_MINUTES</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>{minutes} / {target} session minutes</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>{minutes} / {target} min de sesión</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>{minutes} / {target} min de session</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>FRIENDS_LISTENED_MINUTES</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>{minutes} minutes listened</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>{minutes} minutos escuchados</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>{minutes} minutes écoutées</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>FRIENDS_LISTENING_MINUTES</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Listening minutes</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Minutos escuchados</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Minutes d’écoute</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>FRIENDS_XP_MILESTONE</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>{minutes} min · +{xp} XP</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>{minutes} min · +{xp} XP</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>{minutes} min · +{xp} XP</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>FRIENDS_MILESTONE_REACHED</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Earned</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Conseguido</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Obtenu</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>FRIENDS_MILESTONE_PENDING</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Not yet</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>À atteindre</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>FRIENDS_SESSION_RULE</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Only time actually played counts. After 90 seconds without listening, a new session starts.</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Solo cuenta el tiempo reproducido. Tras 90 segundos sin escuchar, empieza otra sesión.</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Seul le temps réellement lu compte. Après 90 secondes sans écoute, une nouvelle session commence.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(social): unlock and compare original Rockit emblems [KB-36]
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D677"/>
+  <dimension ref="A1:D692"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -14486,6 +14486,336 @@
         </is>
       </c>
     </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGES</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Rockit emblems</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Emblemas Rockit</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Emblèmes Rockit</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_COUNT</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>{count} of {total} earned</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>{count} de {total} conseguidos</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>{count} sur {total} obtenus</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_EARNED</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Unlocked</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Desbloqueado</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Débloqué</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_LOCKED</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Por desbloquear</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>À débloquer</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_COMPARE</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Emblem collections</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Colecciones de emblemas</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Collections d’emblèmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_COMMON</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>{count} earned in common</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>{count} conseguidos en común</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>{count} obtenus en commun</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>FRIENDS_COMPARE_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Compare with your friends</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Comparar con tus amigos</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Comparer avec vos amis</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_IGNITION</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Ignition</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Chispa</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Étincelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_ORBIT</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Orbit</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Órbita</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Orbite</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_GROOVE</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Deep groove</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Surco profundo</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Sillon profond</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_LONGPLAY</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Side B</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Cara B</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Face B</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_ATLAS</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Sound cartographer</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Cartógrafo sonoro</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Cartographe sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VOYAGER</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Interstellar</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Viaje interestelar</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Interstellaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Listen for {minutes} minutes in one session.</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Escucha {minutes} minutos en una sesión.</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Écoutez {minutes} minutes en une session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Accumulate {minutes} verified listening minutes.</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Acumula {minutes} minutos de escucha verificada.</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Cumulez {minutes} minutes d’écoute vérifiées.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(i18n): include shared Friends actions in Excel-generated defaults [KB-34]
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -5650,13 +5650,15 @@
           <t>No results</t>
         </is>
       </c>
-      <c r="C258">
-        <f>_xlfn.TRANSLATE(B258,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D258">
-        <f>_xlfn.TRANSLATE(B258,$B$2,D$2)</f>
-        <v/>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Sin resultados</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Aucun résultat</t>
+        </is>
       </c>
     </row>
     <row r="259">
@@ -8532,6 +8534,7 @@
         <v/>
       </c>
     </row>
+    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(KB-36): expand Rockit emblems across listening and social milestones
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D692"/>
+  <dimension ref="A1:D834"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -14783,17 +14783,17 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Listen for {minutes} minutes in one session.</t>
+          <t>Listen for {target} minutes in one session.</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>Escucha {minutes} minutos en una sesión.</t>
+          <t>Escucha {target} minutos en una sesión.</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Écoutez {minutes} minutes en une session.</t>
+          <t>Écoutez {target} minutes en une session.</t>
         </is>
       </c>
     </row>
@@ -14805,17 +14805,3141 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Accumulate {minutes} verified listening minutes.</t>
+          <t>Accumulate {target} verified listening minutes.</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>Acumula {minutes} minutos de escucha verificada.</t>
+          <t>Acumula {target} minutos de escucha verificada.</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Cumulez {minutes} minutes d’écoute vérifiées.</t>
+          <t>Cumulez {target} minutes d’écoute vérifiées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_01</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Soundcheck</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Prueba de sonido</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_02</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>First riff</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Primer riff</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Premier riff</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_03</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Pulse</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Pulso</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Pulsation</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_04</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Warm-up</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Calentamiento</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Échauffement</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_06</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Takeoff</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Despegue</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Décollage</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_08</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>On repeat</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>En bucle</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>En boucle</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_10</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>The bridge</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>El puente</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Le pont</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_11</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Encore</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Bis</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Rappel</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_13</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Extended mix</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Versión extendida</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Version longue</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_14</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Double album</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Álbum doble</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Double album</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_15</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Main stage</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Escenario principal</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Grande scène</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_16</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Live set</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Directo completo</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Concert complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_17</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Headliner</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Cabeza de cartel</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Tête d’affiche</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_18</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Analog marathon</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Maratón analógico</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Marathon analogique</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_19</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Five-hour odyssey</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Odisea de cinco horas</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Odyssée de cinq heures</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_20</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Endless groove</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Surco infinito</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Sillon sans fin</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_01</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>First resonance</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Primera resonancia</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Première résonance</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_02</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Open ears</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Oídos abiertos</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Oreilles ouvertes</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_03</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Pocket playlist</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Playlist de bolsillo</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Playlist de poche</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_04</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>An hour of sound</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Una hora de sonido</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Une heure de son</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_05</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Tuning in</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Sintonizando</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>À l’écoute</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_06</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Sound traveller</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Viajero sonoro</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Voyageur sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_08</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Ten-hour tape</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Cinta de diez horas</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Cassette de dix heures</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_09</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Personal frequency</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Frecuencia propia</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Fréquence personnelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_11</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Resonance chamber</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Cámara de resonancia</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Chambre de résonance</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_12</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Forty-eight revolutions</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Cuarenta y ocho vueltas</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Quarante-huit tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_13</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Sound explorer</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Explorador sonoro</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Explorateur sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_14</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Hundred-hour horizon</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Horizonte de cien horas</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Horizon de cent heures</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_15</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>A week in sound</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Una semana de sonido</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Une semaine de son</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_16</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>The long wave</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>La onda larga</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>L’onde longue</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_17</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Frequency keeper</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Guardián de frecuencias</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>Gardien des fréquences</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_18</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Five hundred hours</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Quinientas horas</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Cinq cents heures</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_19</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Month of music</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Un mes de música</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>Un mois de musique</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_20</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Thousand-hour club</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Club de las mil horas</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>Club des mille heures</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_21</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Sound observatory</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Observatorio sonoro</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>Observatoire sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_22</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Beyond the dial</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Más allá del dial</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Au-delà du cadran</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_23</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Personal galaxy</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Galaxia propia</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>Galaxie personnelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_24</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Deep-space listener</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Oyente del espacio profundo</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Auditeur de l’espace profond</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TOTAL_25</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>A year in waves</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Un año entre ondas</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Une année dans les ondes</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_01</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>First spin</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Primer giro</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>Premier tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_02</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Five on the deck</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Cinco en el plato</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Cinq sur la platine</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_03</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Ten-track tape</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Cinta de diez temas</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Cassette de dix titres</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_04</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Quarter century</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Cuarto de siglo</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>Quart de siècle</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_05</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Fifty favourites</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Cincuenta escuchas</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Cinquante écoutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_06</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Hundred spins</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Cien vueltas</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Cent tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_07</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Turntable regular</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Habitual del plato</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>Habitué de la platine</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_08</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Five hundred spins</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Quinientas vueltas</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Cinq cents tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_09</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Thousand-track trail</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Mil huellas sonoras</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Mille traces sonores</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_10</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Jukebox keeper</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Guardián de la jukebox</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Gardien du jukebox</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_11</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Setlist archivist</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Archivista de repertorios</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Archiviste des répertoires</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_12</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Five thousand grooves</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Cinco mil surcos</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Cinq mille sillons</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_13</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Recorded history</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Historia grabada</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Histoire enregistrée</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_14</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Five figures</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Cinco cifras</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Cinq chiffres</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_15</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Sound chronicler</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Cronista sonoro</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Chroniqueur sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_16</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Living jukebox</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Jukebox viviente</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Jukebox vivant</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_17</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Fifty thousand echoes</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Cincuenta mil ecos</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Cinquante mille échos</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_18</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Archive without borders</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Archivo sin fronteras</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Archives sans frontières</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_19</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Hundred thousand spins</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Cien mil vueltas</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Cent mille tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_20</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>The eternal turntable</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>El plato eterno</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>La platine éternelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_01</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>First discovery</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Primer descubrimiento</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Première découverte</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_02</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Three new doors</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Tres puertas nuevas</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Trois nouvelles portes</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_03</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Off the beaten track</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Fuera de la ruta</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Hors des sentiers battus</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_04</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Ten directions</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Diez direcciones</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Dix directions</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_05</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Crate digger</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Buscador de vinilos</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Chineur de vinyles</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_06</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Fifty windows</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Cincuenta ventanas</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Cinquante fenêtres</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_07</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Open catalogue</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Catálogo abierto</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Catalogue ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_08</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Two hundred worlds</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Doscientos mundos</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Deux cents mondes</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_09</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Beyond your shelf</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Más allá de tu estantería</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Au-delà de votre étagère</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_10</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Five hundred discoveries</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Quinientos descubrimientos</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Cinq cents découvertes</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_11</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Sound prospector</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Prospector sonoro</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Prospecteur sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_12</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Thousand different grooves</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Mil surcos distintos</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Mille sillons différents</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_13</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Uncharted collection</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Colección inexplorada</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Collection inexplorée</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_14</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Five thousand doors</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Cinco mil puertas</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Cinq mille portes</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_15</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Limitless curiosity</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Curiosidad sin límites</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Curiosité sans limites</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_01</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Back for more</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Volver a por más</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>De retour</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_02</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Three-day rhythm</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Ritmo de tres días</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Rythme de trois jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_03</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Steady beat</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Pulso constante</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Tempo régulier</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_04</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Seven-day groove</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Surco de siete días</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Sillon de sept jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_05</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>A ten-day habit</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Diez días de costumbre</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Dix jours d’habitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_06</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Two-week rhythm</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Ritmo de dos semanas</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Rythme de deux semaines</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_07</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Three-week set</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Sesión de tres semanas</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Session de trois semaines</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_08</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Thirty-day frequency</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Frecuencia de treinta días</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Fréquence de trente jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_09</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Sixty-day pulse</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Pulso de sesenta días</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Pulsation de soixante jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_10</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Hundred-day resonance</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Resonancia de cien días</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Résonance de cent jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_01</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Pass the headphones</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Pasa los auriculares</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Passez le casque</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_02</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Two-way radio</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Radio de ida y vuelta</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Radio bidirectionnelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_03</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Three recommendations</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Tres recomendaciones</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Trois recommandations</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_04</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Small broadcaster</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Pequeña emisora</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Petite station</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_05</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Ten good finds</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Diez buenos hallazgos</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Dix belles trouvailles</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_06</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Music connector</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Conector musical</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Passeur de musique</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_07</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Circle selector</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Selector del círculo</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Sélectionneur du cercle</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_08</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Fifty shared signals</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Cincuenta señales compartidas</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Cinquante signaux partagés</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_09</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Trusted tastemaker</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Prescriptor de confianza</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Prescripteur de confiance</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_10</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>The human radio</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>La radio humana</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>La radio humaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Reach {target} recorded listens.</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Alcanza {target} escuchas registradas.</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Atteignez {target} écoutes enregistrées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Listen to {target} different recordings.</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Escucha {target} grabaciones distintas.</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Écoutez {target} enregistrements différents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_STREAK_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Listen on {target} consecutive days.</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Escucha durante {target} días consecutivos.</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Écoutez pendant {target} jours consécutifs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Share {target} distinct recommendations. Repeating an item to the same friend does not count.</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Comparte {target} recomendaciones distintas. Repetir un envío a la misma persona no suma.</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Partagez {target} recommandations distinctes. Répéter un envoi au même ami ne compte pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_SESSION</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Sesiones</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_TOTAL</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Listening time</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Tiempo de escucha</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Temps d’écoute</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_PLAYS</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Recorded listens</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Escuchas registradas</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Écoutes enregistrées</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_DISCOVERY</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Descubrimientos</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Découvertes</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_STREAK</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Day streaks</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Rachas de días</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Séries de jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_SHARING</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Sharing</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Recomendaciones</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Recommandations</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_EASY</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Facile</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MEDIUM</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_HARD</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Difícil</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Difficile</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_ALL</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>All emblems</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Todos los emblemas</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Tous les emblèmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_ALL_DIFFICULTIES</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>All difficulties</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Todas las dificultades</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Toutes les difficultés</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FILTER_FAMILY</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Filter by family</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Filtrar por familia</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Filtrer par famille</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FILTER_DIFFICULTY</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Filter by difficulty</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Filtrar por dificultad</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Filtrer par difficulté</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FILTER_STATUS</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Filter by status</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Filtrar por estado</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Filtrer par état</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_ALL_STATES</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Earned and locked</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Conseguidos y pendientes</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Obtenus et verrouillés</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SEARCH</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Search emblems</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Buscar emblemas</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Rechercher des emblèmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>{current} / {target}</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>{current} / {target}</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>{current} / {target}</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHOW_ALL</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Explore all {count} emblems</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Explorar los {count} emblemas</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Explorer les {count} emblèmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHOW_FEWER</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Show a summary</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Ver resumen</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Afficher le résumé</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_NO_MATCHES</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>No emblems match these filters.</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>No hay emblemas con estos filtros.</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Aucun emblème ne correspond à ces filtres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_CLEAR_FILTERS</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Clear filters</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Limpiar filtros</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Effacer les filtres</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_TIER</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Collection tier {tier}</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Nivel de colección {tier}</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Palier de collection {tier}</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_RESULTS</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>{count} matching emblems</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>{count} emblemas encontrados</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>{count} emblèmes correspondants</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_01</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Backstage pass</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Pase de backstage</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Pass backstage</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_02</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Power trio</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Power trío</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Power trio</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_03</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Your band</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Tu banda</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Votre groupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_04</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Listening crew</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Comunidad sonora</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Collectif sonore</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_05</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Festival crowd</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Público de festival</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Foule du festival</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_01</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>First frame</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Primer fotograma</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Première image</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_02</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Music in motion</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Música en movimiento</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Musique en mouvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_03</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Director’s cut</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Versión del director</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Version du réalisateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_04</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Front-row screen</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Primera fila</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Premier rang</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_05</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Rockit cinema</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Cine Rockit</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Cinéma Rockit</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_01</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Discover and share</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Descubre y comparte</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Découvrez et partagez</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_02</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Sound scout</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Explorador musical</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Éclaireur musical</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_03</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Taste maker</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Prescriptor musical</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Créateur de tendances</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_04</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Musical crossroads</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Cruce de caminos</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Carrefour musical</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_05</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Rockit ambassador</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Embajador Rockit</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Ambassadeur Rockit</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Amigos</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Amis</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_VIDEOS</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Videos</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Vídeos</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Vidéos</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FAMILY_MIXED</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Discover and share</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Descubre y comparte</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Découvrez et partagez</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Reach {target} mutually accepted friends.</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Alcanza {target} amistades aceptadas por ambas personas.</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Atteignez {target} amitiés acceptées des deux côtés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Complete {target} registered video plays. Audio-only playback is not proof of watching the screen.</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Completa {target} reproducciones registradas de vídeos. No requiere mirar la pantalla.</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Terminez {target} lectures de vidéos enregistrées, sans obligation de regarder l’écran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Reach {target} different recordings listened to and {target} distinct recommendations shared.</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Alcanza {target} grabaciones distintas escuchadas y {target} recomendaciones distintas compartidas.</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Atteignez {target} enregistrements différents écoutés et {target} recommandations distinctes partagées.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(KB-36): localize singular emblem requirements
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D834"/>
+  <dimension ref="A1:D841"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -17907,17 +17907,17 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>Complete {target} registered video plays. Audio-only playback is not proof of watching the screen.</t>
+          <t>Complete {target} registered video plays.</t>
         </is>
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>Completa {target} reproducciones registradas de vídeos. No requiere mirar la pantalla.</t>
+          <t>Completa {target} reproducciones registradas de vídeos.</t>
         </is>
       </c>
       <c r="D833" t="inlineStr">
         <is>
-          <t>Terminez {target} lectures de vidéos enregistrées, sans obligation de regarder l’écran.</t>
+          <t>Terminez {target} lectures de vidéos enregistrées.</t>
         </is>
       </c>
     </row>
@@ -17940,6 +17940,160 @@
       <c r="D834" t="inlineStr">
         <is>
           <t>Atteignez {target} enregistrements différents écoutés et {target} recommandations distinctes partagées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SESSION_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Listen for one minute in one session.</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Escucha un minuto en una sesión.</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Écoutez une minute en une session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_PLAYS_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Complete your first registered listen.</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Completa tu primera escucha registrada.</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Terminez votre première écoute enregistrée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_DISCOVERY_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Listen to your first recording.</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Escucha tu primera grabación.</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Écoutez votre premier enregistrement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_SHARING_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Share your first recommendation.</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Comparte tu primera recomendación.</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Partagez votre première recommandation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_FRIENDS_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Make your first mutually accepted friend.</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Consigue tu primera amistad aceptada por ambas personas.</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Obtenez votre première amitié acceptée des deux côtés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_VIDEOS_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Complete your first registered video play.</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Completa tu primera reproducción registrada de un vídeo.</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>Terminez votre première lecture de vidéo enregistrée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>FRIENDS_BADGE_MIXED_DESCRIPTION_ONE</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Listen to one recording and share one recommendation.</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Escucha una grabación y comparte una recomendación.</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Écoutez un enregistrement et partagez une recommandation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(KB-36): shorten emblem requirements and remove difficulty
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D841"/>
+  <dimension ref="A1:D836"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -14783,17 +14783,17 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Listen for {target} minutes in one session.</t>
+          <t>{target} min in one session</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>Escucha {target} minutos en una sesión.</t>
+          <t>{target} min en una sesión</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Écoutez {target} minutes en une session.</t>
+          <t>{target} min en une session</t>
         </is>
       </c>
     </row>
@@ -14805,17 +14805,17 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Accumulate {target} verified listening minutes.</t>
+          <t>{target} min listened</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>Acumula {target} minutos de escucha verificada.</t>
+          <t>{target} min de escucha</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Cumulez {target} minutes d’écoute vérifiées.</t>
+          <t>{target} min d’écoute</t>
         </is>
       </c>
     </row>
@@ -16895,17 +16895,17 @@
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>Reach {target} recorded listens.</t>
+          <t>{target} recorded listens</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
         <is>
-          <t>Alcanza {target} escuchas registradas.</t>
+          <t>{target} escuchas registradas</t>
         </is>
       </c>
       <c r="D787" t="inlineStr">
         <is>
-          <t>Atteignez {target} écoutes enregistrées.</t>
+          <t>{target} écoutes enregistrées</t>
         </is>
       </c>
     </row>
@@ -16917,17 +16917,17 @@
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>Listen to {target} different recordings.</t>
+          <t>{target} different recordings</t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
         <is>
-          <t>Escucha {target} grabaciones distintas.</t>
+          <t>{target} grabaciones distintas</t>
         </is>
       </c>
       <c r="D788" t="inlineStr">
         <is>
-          <t>Écoutez {target} enregistrements différents.</t>
+          <t>{target} enregistrements différents</t>
         </is>
       </c>
     </row>
@@ -16939,17 +16939,17 @@
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>Listen on {target} consecutive days.</t>
+          <t>{target} consecutive days</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>Escucha durante {target} días consecutivos.</t>
+          <t>{target} días seguidos</t>
         </is>
       </c>
       <c r="D789" t="inlineStr">
         <is>
-          <t>Écoutez pendant {target} jours consécutifs.</t>
+          <t>{target} jours consécutifs</t>
         </is>
       </c>
     </row>
@@ -16961,17 +16961,17 @@
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>Share {target} distinct recommendations. Repeating an item to the same friend does not count.</t>
+          <t>{target} distinct recommendations</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
         <is>
-          <t>Comparte {target} recomendaciones distintas. Repetir un envío a la misma persona no suma.</t>
+          <t>{target} recomendaciones distintas</t>
         </is>
       </c>
       <c r="D790" t="inlineStr">
         <is>
-          <t>Partagez {target} recommandations distinctes. Répéter un envoi au même ami ne compte pas.</t>
+          <t>{target} recommandations distinctes</t>
         </is>
       </c>
     </row>
@@ -17110,990 +17110,880 @@
     <row r="797">
       <c r="A797" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_EASY</t>
+          <t>FRIENDS_BADGE_ALL</t>
         </is>
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>All emblems</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Todos los emblemas</t>
         </is>
       </c>
       <c r="D797" t="inlineStr">
         <is>
-          <t>Facile</t>
+          <t>Tous les emblèmes</t>
         </is>
       </c>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MEDIUM</t>
+          <t>FRIENDS_BADGE_FILTER_FAMILY</t>
         </is>
       </c>
       <c r="B798" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Filter by family</t>
         </is>
       </c>
       <c r="C798" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Filtrar por familia</t>
         </is>
       </c>
       <c r="D798" t="inlineStr">
         <is>
-          <t>Moyenne</t>
+          <t>Filtrer par famille</t>
         </is>
       </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_HARD</t>
+          <t>FRIENDS_BADGE_FILTER_STATUS</t>
         </is>
       </c>
       <c r="B799" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Filter by status</t>
         </is>
       </c>
       <c r="C799" t="inlineStr">
         <is>
-          <t>Difícil</t>
+          <t>Filtrar por estado</t>
         </is>
       </c>
       <c r="D799" t="inlineStr">
         <is>
-          <t>Difficile</t>
+          <t>Filtrer par état</t>
         </is>
       </c>
     </row>
     <row r="800">
       <c r="A800" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_ALL</t>
+          <t>FRIENDS_BADGE_ALL_STATES</t>
         </is>
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>All emblems</t>
+          <t>Earned and locked</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Todos los emblemas</t>
+          <t>Conseguidos y pendientes</t>
         </is>
       </c>
       <c r="D800" t="inlineStr">
         <is>
-          <t>Tous les emblèmes</t>
+          <t>Obtenus et verrouillés</t>
         </is>
       </c>
     </row>
     <row r="801">
       <c r="A801" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_ALL_DIFFICULTIES</t>
+          <t>FRIENDS_BADGE_SEARCH</t>
         </is>
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>All difficulties</t>
+          <t>Search emblems</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
         <is>
-          <t>Todas las dificultades</t>
+          <t>Buscar emblemas</t>
         </is>
       </c>
       <c r="D801" t="inlineStr">
         <is>
-          <t>Toutes les difficultés</t>
+          <t>Rechercher des emblèmes</t>
         </is>
       </c>
     </row>
     <row r="802">
       <c r="A802" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FILTER_FAMILY</t>
+          <t>FRIENDS_BADGE_PROGRESS</t>
         </is>
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>Filter by family</t>
+          <t>{current} / {target}</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
         <is>
-          <t>Filtrar por familia</t>
+          <t>{current} / {target}</t>
         </is>
       </c>
       <c r="D802" t="inlineStr">
         <is>
-          <t>Filtrer par famille</t>
+          <t>{current} / {target}</t>
         </is>
       </c>
     </row>
     <row r="803">
       <c r="A803" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FILTER_DIFFICULTY</t>
+          <t>FRIENDS_BADGE_SHOW_ALL</t>
         </is>
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Filter by difficulty</t>
+          <t>Explore all {count} emblems</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>Filtrar por dificultad</t>
+          <t>Explorar los {count} emblemas</t>
         </is>
       </c>
       <c r="D803" t="inlineStr">
         <is>
-          <t>Filtrer par difficulté</t>
+          <t>Explorer les {count} emblèmes</t>
         </is>
       </c>
     </row>
     <row r="804">
       <c r="A804" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FILTER_STATUS</t>
+          <t>FRIENDS_BADGE_SHOW_FEWER</t>
         </is>
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>Filter by status</t>
+          <t>Show a summary</t>
         </is>
       </c>
       <c r="C804" t="inlineStr">
         <is>
-          <t>Filtrar por estado</t>
+          <t>Ver resumen</t>
         </is>
       </c>
       <c r="D804" t="inlineStr">
         <is>
-          <t>Filtrer par état</t>
+          <t>Afficher le résumé</t>
         </is>
       </c>
     </row>
     <row r="805">
       <c r="A805" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_ALL_STATES</t>
+          <t>FRIENDS_BADGE_NO_MATCHES</t>
         </is>
       </c>
       <c r="B805" t="inlineStr">
         <is>
-          <t>Earned and locked</t>
+          <t>No emblems match these filters.</t>
         </is>
       </c>
       <c r="C805" t="inlineStr">
         <is>
-          <t>Conseguidos y pendientes</t>
+          <t>No hay emblemas con estos filtros.</t>
         </is>
       </c>
       <c r="D805" t="inlineStr">
         <is>
-          <t>Obtenus et verrouillés</t>
+          <t>Aucun emblème ne correspond à ces filtres.</t>
         </is>
       </c>
     </row>
     <row r="806">
       <c r="A806" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_SEARCH</t>
+          <t>FRIENDS_BADGE_CLEAR_FILTERS</t>
         </is>
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>Search emblems</t>
+          <t>Clear filters</t>
         </is>
       </c>
       <c r="C806" t="inlineStr">
         <is>
-          <t>Buscar emblemas</t>
+          <t>Limpiar filtros</t>
         </is>
       </c>
       <c r="D806" t="inlineStr">
         <is>
-          <t>Rechercher des emblèmes</t>
+          <t>Effacer les filtres</t>
         </is>
       </c>
     </row>
     <row r="807">
       <c r="A807" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_PROGRESS</t>
+          <t>FRIENDS_BADGE_TIER</t>
         </is>
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>{current} / {target}</t>
+          <t>Collection tier {tier}</t>
         </is>
       </c>
       <c r="C807" t="inlineStr">
         <is>
-          <t>{current} / {target}</t>
+          <t>Nivel de colección {tier}</t>
         </is>
       </c>
       <c r="D807" t="inlineStr">
         <is>
-          <t>{current} / {target}</t>
+          <t>Palier de collection {tier}</t>
         </is>
       </c>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_SHOW_ALL</t>
+          <t>FRIENDS_BADGE_RESULTS</t>
         </is>
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Explore all {count} emblems</t>
+          <t>{count} matching emblems</t>
         </is>
       </c>
       <c r="C808" t="inlineStr">
         <is>
-          <t>Explorar los {count} emblemas</t>
+          <t>{count} emblemas encontrados</t>
         </is>
       </c>
       <c r="D808" t="inlineStr">
         <is>
-          <t>Explorer les {count} emblèmes</t>
+          <t>{count} emblèmes correspondants</t>
         </is>
       </c>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_SHOW_FEWER</t>
+          <t>FRIENDS_BADGE_FRIENDS_01</t>
         </is>
       </c>
       <c r="B809" t="inlineStr">
         <is>
-          <t>Show a summary</t>
+          <t>Backstage pass</t>
         </is>
       </c>
       <c r="C809" t="inlineStr">
         <is>
-          <t>Ver resumen</t>
+          <t>Pase de backstage</t>
         </is>
       </c>
       <c r="D809" t="inlineStr">
         <is>
-          <t>Afficher le résumé</t>
+          <t>Pass backstage</t>
         </is>
       </c>
     </row>
     <row r="810">
       <c r="A810" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_NO_MATCHES</t>
+          <t>FRIENDS_BADGE_FRIENDS_02</t>
         </is>
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>No emblems match these filters.</t>
+          <t>Power trio</t>
         </is>
       </c>
       <c r="C810" t="inlineStr">
         <is>
-          <t>No hay emblemas con estos filtros.</t>
+          <t>Power trío</t>
         </is>
       </c>
       <c r="D810" t="inlineStr">
         <is>
-          <t>Aucun emblème ne correspond à ces filtres.</t>
+          <t>Power trio</t>
         </is>
       </c>
     </row>
     <row r="811">
       <c r="A811" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_CLEAR_FILTERS</t>
+          <t>FRIENDS_BADGE_FRIENDS_03</t>
         </is>
       </c>
       <c r="B811" t="inlineStr">
         <is>
-          <t>Clear filters</t>
+          <t>Your band</t>
         </is>
       </c>
       <c r="C811" t="inlineStr">
         <is>
-          <t>Limpiar filtros</t>
+          <t>Tu banda</t>
         </is>
       </c>
       <c r="D811" t="inlineStr">
         <is>
-          <t>Effacer les filtres</t>
+          <t>Votre groupe</t>
         </is>
       </c>
     </row>
     <row r="812">
       <c r="A812" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_TIER</t>
+          <t>FRIENDS_BADGE_FRIENDS_04</t>
         </is>
       </c>
       <c r="B812" t="inlineStr">
         <is>
-          <t>Collection tier {tier}</t>
+          <t>Listening crew</t>
         </is>
       </c>
       <c r="C812" t="inlineStr">
         <is>
-          <t>Nivel de colección {tier}</t>
+          <t>Comunidad sonora</t>
         </is>
       </c>
       <c r="D812" t="inlineStr">
         <is>
-          <t>Palier de collection {tier}</t>
+          <t>Collectif sonore</t>
         </is>
       </c>
     </row>
     <row r="813">
       <c r="A813" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_RESULTS</t>
+          <t>FRIENDS_BADGE_FRIENDS_05</t>
         </is>
       </c>
       <c r="B813" t="inlineStr">
         <is>
-          <t>{count} matching emblems</t>
+          <t>Festival crowd</t>
         </is>
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>{count} emblemas encontrados</t>
+          <t>Público de festival</t>
         </is>
       </c>
       <c r="D813" t="inlineStr">
         <is>
-          <t>{count} emblèmes correspondants</t>
+          <t>Foule du festival</t>
         </is>
       </c>
     </row>
     <row r="814">
       <c r="A814" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FRIENDS_01</t>
+          <t>FRIENDS_BADGE_VIDEOS_01</t>
         </is>
       </c>
       <c r="B814" t="inlineStr">
         <is>
-          <t>Backstage pass</t>
+          <t>First frame</t>
         </is>
       </c>
       <c r="C814" t="inlineStr">
         <is>
-          <t>Pase de backstage</t>
+          <t>Primer fotograma</t>
         </is>
       </c>
       <c r="D814" t="inlineStr">
         <is>
-          <t>Pass backstage</t>
+          <t>Première image</t>
         </is>
       </c>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FRIENDS_02</t>
+          <t>FRIENDS_BADGE_VIDEOS_02</t>
         </is>
       </c>
       <c r="B815" t="inlineStr">
         <is>
-          <t>Power trio</t>
+          <t>Music in motion</t>
         </is>
       </c>
       <c r="C815" t="inlineStr">
         <is>
-          <t>Power trío</t>
+          <t>Música en movimiento</t>
         </is>
       </c>
       <c r="D815" t="inlineStr">
         <is>
-          <t>Power trio</t>
+          <t>Musique en mouvement</t>
         </is>
       </c>
     </row>
     <row r="816">
       <c r="A816" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FRIENDS_03</t>
+          <t>FRIENDS_BADGE_VIDEOS_03</t>
         </is>
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>Your band</t>
+          <t>Director’s cut</t>
         </is>
       </c>
       <c r="C816" t="inlineStr">
         <is>
-          <t>Tu banda</t>
+          <t>Versión del director</t>
         </is>
       </c>
       <c r="D816" t="inlineStr">
         <is>
-          <t>Votre groupe</t>
+          <t>Version du réalisateur</t>
         </is>
       </c>
     </row>
     <row r="817">
       <c r="A817" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FRIENDS_04</t>
+          <t>FRIENDS_BADGE_VIDEOS_04</t>
         </is>
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>Listening crew</t>
+          <t>Front-row screen</t>
         </is>
       </c>
       <c r="C817" t="inlineStr">
         <is>
-          <t>Comunidad sonora</t>
+          <t>Primera fila</t>
         </is>
       </c>
       <c r="D817" t="inlineStr">
         <is>
-          <t>Collectif sonore</t>
+          <t>Premier rang</t>
         </is>
       </c>
     </row>
     <row r="818">
       <c r="A818" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FRIENDS_05</t>
+          <t>FRIENDS_BADGE_VIDEOS_05</t>
         </is>
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>Festival crowd</t>
+          <t>Rockit cinema</t>
         </is>
       </c>
       <c r="C818" t="inlineStr">
         <is>
-          <t>Público de festival</t>
+          <t>Cine Rockit</t>
         </is>
       </c>
       <c r="D818" t="inlineStr">
         <is>
-          <t>Foule du festival</t>
+          <t>Cinéma Rockit</t>
         </is>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_VIDEOS_01</t>
+          <t>FRIENDS_BADGE_MIXED_01</t>
         </is>
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>First frame</t>
+          <t>Discover and share</t>
         </is>
       </c>
       <c r="C819" t="inlineStr">
         <is>
-          <t>Primer fotograma</t>
+          <t>Descubre y comparte</t>
         </is>
       </c>
       <c r="D819" t="inlineStr">
         <is>
-          <t>Première image</t>
+          <t>Découvrez et partagez</t>
         </is>
       </c>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_VIDEOS_02</t>
+          <t>FRIENDS_BADGE_MIXED_02</t>
         </is>
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>Music in motion</t>
+          <t>Sound scout</t>
         </is>
       </c>
       <c r="C820" t="inlineStr">
         <is>
-          <t>Música en movimiento</t>
+          <t>Explorador musical</t>
         </is>
       </c>
       <c r="D820" t="inlineStr">
         <is>
-          <t>Musique en mouvement</t>
+          <t>Éclaireur musical</t>
         </is>
       </c>
     </row>
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_VIDEOS_03</t>
+          <t>FRIENDS_BADGE_MIXED_03</t>
         </is>
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>Director’s cut</t>
+          <t>Taste maker</t>
         </is>
       </c>
       <c r="C821" t="inlineStr">
         <is>
-          <t>Versión del director</t>
+          <t>Prescriptor musical</t>
         </is>
       </c>
       <c r="D821" t="inlineStr">
         <is>
-          <t>Version du réalisateur</t>
+          <t>Créateur de tendances</t>
         </is>
       </c>
     </row>
     <row r="822">
       <c r="A822" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_VIDEOS_04</t>
+          <t>FRIENDS_BADGE_MIXED_04</t>
         </is>
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>Front-row screen</t>
+          <t>Musical crossroads</t>
         </is>
       </c>
       <c r="C822" t="inlineStr">
         <is>
-          <t>Primera fila</t>
+          <t>Cruce de caminos</t>
         </is>
       </c>
       <c r="D822" t="inlineStr">
         <is>
-          <t>Premier rang</t>
+          <t>Carrefour musical</t>
         </is>
       </c>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_VIDEOS_05</t>
+          <t>FRIENDS_BADGE_MIXED_05</t>
         </is>
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Rockit cinema</t>
+          <t>Rockit ambassador</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
         <is>
-          <t>Cine Rockit</t>
+          <t>Embajador Rockit</t>
         </is>
       </c>
       <c r="D823" t="inlineStr">
         <is>
-          <t>Cinéma Rockit</t>
+          <t>Ambassadeur Rockit</t>
         </is>
       </c>
     </row>
     <row r="824">
       <c r="A824" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MIXED_01</t>
+          <t>FRIENDS_BADGE_FAMILY_FRIENDS</t>
         </is>
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Discover and share</t>
+          <t>Friends</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
         <is>
-          <t>Descubre y comparte</t>
+          <t>Amigos</t>
         </is>
       </c>
       <c r="D824" t="inlineStr">
         <is>
-          <t>Découvrez et partagez</t>
+          <t>Amis</t>
         </is>
       </c>
     </row>
     <row r="825">
       <c r="A825" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MIXED_02</t>
+          <t>FRIENDS_BADGE_FAMILY_VIDEOS</t>
         </is>
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Sound scout</t>
+          <t>Videos</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>Explorador musical</t>
+          <t>Vídeos</t>
         </is>
       </c>
       <c r="D825" t="inlineStr">
         <is>
-          <t>Éclaireur musical</t>
+          <t>Vidéos</t>
         </is>
       </c>
     </row>
     <row r="826">
       <c r="A826" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MIXED_03</t>
+          <t>FRIENDS_BADGE_FAMILY_MIXED</t>
         </is>
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Taste maker</t>
+          <t>Discover and share</t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>Prescriptor musical</t>
+          <t>Descubre y comparte</t>
         </is>
       </c>
       <c r="D826" t="inlineStr">
         <is>
-          <t>Créateur de tendances</t>
+          <t>Découvrez et partagez</t>
         </is>
       </c>
     </row>
     <row r="827">
       <c r="A827" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MIXED_04</t>
+          <t>FRIENDS_BADGE_FRIENDS_DESCRIPTION</t>
         </is>
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>Musical crossroads</t>
+          <t>{target} mutual friends</t>
         </is>
       </c>
       <c r="C827" t="inlineStr">
         <is>
-          <t>Cruce de caminos</t>
+          <t>{target} amigos</t>
         </is>
       </c>
       <c r="D827" t="inlineStr">
         <is>
-          <t>Carrefour musical</t>
+          <t>{target} amis</t>
         </is>
       </c>
     </row>
     <row r="828">
       <c r="A828" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MIXED_05</t>
+          <t>FRIENDS_BADGE_VIDEOS_DESCRIPTION</t>
         </is>
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Rockit ambassador</t>
+          <t>{target} completed video plays</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
         <is>
-          <t>Embajador Rockit</t>
+          <t>{target} vídeos reproducidos</t>
         </is>
       </c>
       <c r="D828" t="inlineStr">
         <is>
-          <t>Ambassadeur Rockit</t>
+          <t>{target} vidéos lues</t>
         </is>
       </c>
     </row>
     <row r="829">
       <c r="A829" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FAMILY_FRIENDS</t>
+          <t>FRIENDS_BADGE_MIXED_DESCRIPTION</t>
         </is>
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Friends</t>
+          <t>{target} different recordings and {target} distinct recommendations</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>Amigos</t>
+          <t>{target} grabaciones distintas y {target} recomendaciones distintas</t>
         </is>
       </c>
       <c r="D829" t="inlineStr">
         <is>
-          <t>Amis</t>
+          <t>{target} enregistrements différents et {target} recommandations distinctes</t>
         </is>
       </c>
     </row>
     <row r="830">
       <c r="A830" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FAMILY_VIDEOS</t>
+          <t>FRIENDS_BADGE_SESSION_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Listen for one minute in one session.</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">
         <is>
-          <t>Vídeos</t>
+          <t>Escucha un minuto en una sesión.</t>
         </is>
       </c>
       <c r="D830" t="inlineStr">
         <is>
-          <t>Vidéos</t>
+          <t>Écoutez une minute en une session.</t>
         </is>
       </c>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FAMILY_MIXED</t>
+          <t>FRIENDS_BADGE_PLAYS_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>Discover and share</t>
+          <t>{target} recorded listen</t>
         </is>
       </c>
       <c r="C831" t="inlineStr">
         <is>
-          <t>Descubre y comparte</t>
+          <t>{target} escucha registrada</t>
         </is>
       </c>
       <c r="D831" t="inlineStr">
         <is>
-          <t>Découvrez et partagez</t>
+          <t>{target} écoute enregistrée</t>
         </is>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_FRIENDS_DESCRIPTION</t>
+          <t>FRIENDS_BADGE_DISCOVERY_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>Reach {target} mutually accepted friends.</t>
+          <t>{target} different recording</t>
         </is>
       </c>
       <c r="C832" t="inlineStr">
         <is>
-          <t>Alcanza {target} amistades aceptadas por ambas personas.</t>
+          <t>{target} grabación distinta</t>
         </is>
       </c>
       <c r="D832" t="inlineStr">
         <is>
-          <t>Atteignez {target} amitiés acceptées des deux côtés.</t>
+          <t>{target} enregistrement différent</t>
         </is>
       </c>
     </row>
     <row r="833">
       <c r="A833" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_VIDEOS_DESCRIPTION</t>
+          <t>FRIENDS_BADGE_SHARING_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>Complete {target} registered video plays.</t>
+          <t>{target} distinct recommendation</t>
         </is>
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>Completa {target} reproducciones registradas de vídeos.</t>
+          <t>{target} recomendación distinta</t>
         </is>
       </c>
       <c r="D833" t="inlineStr">
         <is>
-          <t>Terminez {target} lectures de vidéos enregistrées.</t>
+          <t>{target} recommandation distincte</t>
         </is>
       </c>
     </row>
     <row r="834">
       <c r="A834" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_MIXED_DESCRIPTION</t>
+          <t>FRIENDS_BADGE_FRIENDS_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>Reach {target} different recordings listened to and {target} distinct recommendations shared.</t>
+          <t>{target} mutual friend</t>
         </is>
       </c>
       <c r="C834" t="inlineStr">
         <is>
-          <t>Alcanza {target} grabaciones distintas escuchadas y {target} recomendaciones distintas compartidas.</t>
+          <t>{target} amigo</t>
         </is>
       </c>
       <c r="D834" t="inlineStr">
         <is>
-          <t>Atteignez {target} enregistrements différents écoutés et {target} recommandations distinctes partagées.</t>
+          <t>{target} ami</t>
         </is>
       </c>
     </row>
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_SESSION_DESCRIPTION_ONE</t>
+          <t>FRIENDS_BADGE_VIDEOS_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Listen for one minute in one session.</t>
+          <t>{target} completed video play</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>Escucha un minuto en una sesión.</t>
+          <t>{target} vídeo reproducido</t>
         </is>
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>Écoutez une minute en une session.</t>
+          <t>{target} vidéo lue</t>
         </is>
       </c>
     </row>
     <row r="836">
       <c r="A836" t="inlineStr">
         <is>
-          <t>FRIENDS_BADGE_PLAYS_DESCRIPTION_ONE</t>
+          <t>FRIENDS_BADGE_MIXED_DESCRIPTION_ONE</t>
         </is>
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>Complete your first registered listen.</t>
+          <t>{target} recording and {target} recommendation</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
         <is>
-          <t>Completa tu primera escucha registrada.</t>
+          <t>{target} grabación y {target} recomendación</t>
         </is>
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>Terminez votre première écoute enregistrée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="837">
-      <c r="A837" t="inlineStr">
-        <is>
-          <t>FRIENDS_BADGE_DISCOVERY_DESCRIPTION_ONE</t>
-        </is>
-      </c>
-      <c r="B837" t="inlineStr">
-        <is>
-          <t>Listen to your first recording.</t>
-        </is>
-      </c>
-      <c r="C837" t="inlineStr">
-        <is>
-          <t>Escucha tu primera grabación.</t>
-        </is>
-      </c>
-      <c r="D837" t="inlineStr">
-        <is>
-          <t>Écoutez votre premier enregistrement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="838">
-      <c r="A838" t="inlineStr">
-        <is>
-          <t>FRIENDS_BADGE_SHARING_DESCRIPTION_ONE</t>
-        </is>
-      </c>
-      <c r="B838" t="inlineStr">
-        <is>
-          <t>Share your first recommendation.</t>
-        </is>
-      </c>
-      <c r="C838" t="inlineStr">
-        <is>
-          <t>Comparte tu primera recomendación.</t>
-        </is>
-      </c>
-      <c r="D838" t="inlineStr">
-        <is>
-          <t>Partagez votre première recommandation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="839">
-      <c r="A839" t="inlineStr">
-        <is>
-          <t>FRIENDS_BADGE_FRIENDS_DESCRIPTION_ONE</t>
-        </is>
-      </c>
-      <c r="B839" t="inlineStr">
-        <is>
-          <t>Make your first mutually accepted friend.</t>
-        </is>
-      </c>
-      <c r="C839" t="inlineStr">
-        <is>
-          <t>Consigue tu primera amistad aceptada por ambas personas.</t>
-        </is>
-      </c>
-      <c r="D839" t="inlineStr">
-        <is>
-          <t>Obtenez votre première amitié acceptée des deux côtés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="840">
-      <c r="A840" t="inlineStr">
-        <is>
-          <t>FRIENDS_BADGE_VIDEOS_DESCRIPTION_ONE</t>
-        </is>
-      </c>
-      <c r="B840" t="inlineStr">
-        <is>
-          <t>Complete your first registered video play.</t>
-        </is>
-      </c>
-      <c r="C840" t="inlineStr">
-        <is>
-          <t>Completa tu primera reproducción registrada de un vídeo.</t>
-        </is>
-      </c>
-      <c r="D840" t="inlineStr">
-        <is>
-          <t>Terminez votre première lecture de vidéo enregistrée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="841">
-      <c r="A841" t="inlineStr">
-        <is>
-          <t>FRIENDS_BADGE_MIXED_DESCRIPTION_ONE</t>
-        </is>
-      </c>
-      <c r="B841" t="inlineStr">
-        <is>
-          <t>Listen to one recording and share one recommendation.</t>
-        </is>
-      </c>
-      <c r="C841" t="inlineStr">
-        <is>
-          <t>Escucha una grabación y comparte una recomendación.</t>
-        </is>
-      </c>
-      <c r="D841" t="inlineStr">
-        <is>
-          <t>Écoutez un enregistrement et partagez une recommandation.</t>
+          <t>{target} enregistrement et {target} recommandation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(KB-36): align singular requirement and Kanban summary
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -17841,17 +17841,17 @@
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>Listen for one minute in one session.</t>
+          <t>{target} min in one session</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">
         <is>
-          <t>Escucha un minuto en una sesión.</t>
+          <t>{target} min en una sesión</t>
         </is>
       </c>
       <c r="D830" t="inlineStr">
         <is>
-          <t>Écoutez une minute en une session.</t>
+          <t>{target} min en une session</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(KB-20): complete Home and media-menu vocabulary translations
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -435,7 +435,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -524,13 +524,15 @@
           <t>Add list to queue randomly</t>
         </is>
       </c>
-      <c r="C4">
-        <f>_xlfn.TRANSLATE(B4,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D4">
-        <f>_xlfn.TRANSLATE(B4,$B$2,D$2)</f>
-        <v/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Añadir lista aleatoriamente a la cola</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ajouter la liste aléatoirement à la file</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -544,13 +546,15 @@
           <t>Add list to bottom of queue</t>
         </is>
       </c>
-      <c r="C5">
-        <f>_xlfn.TRANSLATE(B5,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D5">
-        <f>_xlfn.TRANSLATE(B5,$B$2,D$2)</f>
-        <v/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Añadir lista al final de la cola</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ajouter la liste en fin de file</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -564,13 +568,15 @@
           <t>Add list to queue</t>
         </is>
       </c>
-      <c r="C6">
-        <f>_xlfn.TRANSLATE(B6,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>_xlfn.TRANSLATE(B6,$B$2,D$2)</f>
-        <v/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Añadir lista a la cola</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ajouter la liste à la file</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -626,13 +632,15 @@
           <t>Add song to queue</t>
         </is>
       </c>
-      <c r="C9">
-        <f>_xlfn.TRANSLATE(B9,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>_xlfn.TRANSLATE(B9,$B$2,D$2)</f>
-        <v/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Añadir canción a la cola</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ajouter le morceau à la file</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2560,13 +2568,15 @@
           <t>Carousel navigation</t>
         </is>
       </c>
-      <c r="C105">
-        <f>_xlfn.TRANSLATE(B105,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D105">
-        <f>_xlfn.TRANSLATE(B105,$B$2,D$2)</f>
-        <v/>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Navegación del carrusel</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Navigation du carrousel</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -2620,13 +2630,15 @@
           <t>Click to download</t>
         </is>
       </c>
-      <c r="C108">
-        <f>_xlfn.TRANSLATE(B108,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D108">
-        <f>_xlfn.TRANSLATE(B108,$B$2,D$2)</f>
-        <v/>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Pulsa para descargar</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Appuyez pour télécharger</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -2864,13 +2876,15 @@
           <t>Delete error</t>
         </is>
       </c>
-      <c r="C120">
-        <f>_xlfn.TRANSLATE(B120,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D120">
-        <f>_xlfn.TRANSLATE(B120,$B$2,D$2)</f>
-        <v/>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>No se ha podido eliminar</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Impossible de supprimer</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -2884,13 +2898,15 @@
           <t>Delete success</t>
         </is>
       </c>
-      <c r="C121">
-        <f>_xlfn.TRANSLATE(B121,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D121">
-        <f>_xlfn.TRANSLATE(B121,$B$2,D$2)</f>
-        <v/>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Eliminado correctamente</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Suppression effectuée</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -3070,13 +3086,15 @@
           <t>Download list to device</t>
         </is>
       </c>
-      <c r="C130">
-        <f>_xlfn.TRANSLATE(B130,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D130">
-        <f>_xlfn.TRANSLATE(B130,$B$2,D$2)</f>
-        <v/>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Descargar lista en el dispositivo</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Télécharger la liste sur cet appareil</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -3090,13 +3108,15 @@
           <t>Download list to server</t>
         </is>
       </c>
-      <c r="C131">
-        <f>_xlfn.TRANSLATE(B131,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D131">
-        <f>_xlfn.TRANSLATE(B131,$B$2,D$2)</f>
-        <v/>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Descargar lista en el servidor</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Télécharger la liste sur le serveur</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -3276,13 +3296,15 @@
           <t>Downloading</t>
         </is>
       </c>
-      <c r="C140">
-        <f>_xlfn.TRANSLATE(B140,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D140">
-        <f>_xlfn.TRANSLATE(B140,$B$2,D$2)</f>
-        <v/>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Descargando</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Téléchargement en cours</t>
+        </is>
       </c>
     </row>
     <row r="141">
@@ -3356,13 +3378,15 @@
           <t>Edit metadata</t>
         </is>
       </c>
-      <c r="C144">
-        <f>_xlfn.TRANSLATE(B144,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D144">
-        <f>_xlfn.TRANSLATE(B144,$B$2,D$2)</f>
-        <v/>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Editar metadatos</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Modifier les métadonnées</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -3736,13 +3760,15 @@
           <t>Error creating your new playlist</t>
         </is>
       </c>
-      <c r="C163">
-        <f>_xlfn.TRANSLATE(B163,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D163">
-        <f>_xlfn.TRANSLATE(B163,$B$2,D$2)</f>
-        <v/>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>No se ha podido crear la playlist</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Impossible de créer la playlist</t>
+        </is>
       </c>
     </row>
     <row r="164">
@@ -4138,13 +4164,15 @@
           <t>Featured songs</t>
         </is>
       </c>
-      <c r="C183">
-        <f>_xlfn.TRANSLATE(B183,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D183">
-        <f>_xlfn.TRANSLATE(B183,$B$2,D$2)</f>
-        <v/>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Canciones destacadas</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Morceaux à la une</t>
+        </is>
       </c>
     </row>
     <row r="184">
@@ -4406,13 +4434,15 @@
           <t>Go to album</t>
         </is>
       </c>
-      <c r="C196">
-        <f>_xlfn.TRANSLATE(B196,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D196">
-        <f>_xlfn.TRANSLATE(B196,$B$2,D$2)</f>
-        <v/>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Ir al álbum</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Voir l’album</t>
+        </is>
       </c>
     </row>
     <row r="197">
@@ -4426,13 +4456,15 @@
           <t>Go to artist</t>
         </is>
       </c>
-      <c r="C197">
-        <f>_xlfn.TRANSLATE(B197,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D197">
-        <f>_xlfn.TRANSLATE(B197,$B$2,D$2)</f>
-        <v/>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Ir al artista</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Voir l’artiste</t>
+        </is>
       </c>
     </row>
     <row r="198">
@@ -4546,13 +4578,15 @@
           <t>Home highlights</t>
         </is>
       </c>
-      <c r="C203">
-        <f>_xlfn.TRANSLATE(B203,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D203">
-        <f>_xlfn.TRANSLATE(B203,$B$2,D$2)</f>
-        <v/>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Destacados del inicio</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>À la une</t>
+        </is>
       </c>
     </row>
     <row r="204">
@@ -4566,13 +4600,15 @@
           <t>Listen to</t>
         </is>
       </c>
-      <c r="C204">
-        <f>_xlfn.TRANSLATE(B204,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D204">
-        <f>_xlfn.TRANSLATE(B204,$B$2,D$2)</f>
-        <v/>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Escucha</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Écoutez</t>
+        </is>
       </c>
     </row>
     <row r="205">
@@ -4586,13 +4622,15 @@
           <t>min this week</t>
         </is>
       </c>
-      <c r="C205">
-        <f>_xlfn.TRANSLATE(B205,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D205">
-        <f>_xlfn.TRANSLATE(B205,$B$2,D$2)</f>
-        <v/>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>min esta semana</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>min cette semaine</t>
+        </is>
       </c>
     </row>
     <row r="206">
@@ -4606,13 +4644,15 @@
           <t>days in a row</t>
         </is>
       </c>
-      <c r="C206">
-        <f>_xlfn.TRANSLATE(B206,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D206">
-        <f>_xlfn.TRANSLATE(B206,$B$2,D$2)</f>
-        <v/>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>días seguidos</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>jours consécutifs</t>
+        </is>
       </c>
     </row>
     <row r="207">
@@ -4626,13 +4666,15 @@
           <t>Your music awaits</t>
         </is>
       </c>
-      <c r="C207">
-        <f>_xlfn.TRANSLATE(B207,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D207">
-        <f>_xlfn.TRANSLATE(B207,$B$2,D$2)</f>
-        <v/>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Tu música te espera</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Votre musique vous attend</t>
+        </is>
       </c>
     </row>
     <row r="208">
@@ -5830,13 +5872,15 @@
           <t>Open list</t>
         </is>
       </c>
-      <c r="C267">
-        <f>_xlfn.TRANSLATE(B267,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D267">
-        <f>_xlfn.TRANSLATE(B267,$B$2,D$2)</f>
-        <v/>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Abrir lista</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Ouvrir la liste</t>
+        </is>
       </c>
     </row>
     <row r="268">
@@ -6216,13 +6260,15 @@
           <t>Play list</t>
         </is>
       </c>
-      <c r="C286">
-        <f>_xlfn.TRANSLATE(B286,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D286">
-        <f>_xlfn.TRANSLATE(B286,$B$2,D$2)</f>
-        <v/>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Reproducir lista</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Lire la liste</t>
+        </is>
       </c>
     </row>
     <row r="287">
@@ -6806,13 +6852,15 @@
           <t>Remove from playlist</t>
         </is>
       </c>
-      <c r="C315">
-        <f>_xlfn.TRANSLATE(B315,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D315">
-        <f>_xlfn.TRANSLATE(B315,$B$2,D$2)</f>
-        <v/>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Quitar de la playlist</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Retirer de la playlist</t>
+        </is>
       </c>
     </row>
     <row r="316">
@@ -6826,13 +6874,15 @@
           <t>Remove from queue</t>
         </is>
       </c>
-      <c r="C316">
-        <f>_xlfn.TRANSLATE(B316,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D316">
-        <f>_xlfn.TRANSLATE(B316,$B$2,D$2)</f>
-        <v/>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Quitar de la cola</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Retirer de la file</t>
+        </is>
       </c>
     </row>
     <row r="317">
@@ -6846,13 +6896,15 @@
           <t>Remove from offline</t>
         </is>
       </c>
-      <c r="C317">
-        <f>_xlfn.TRANSLATE($B317,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D317">
-        <f>_xlfn.TRANSLATE($B317,$B$2,D$2)</f>
-        <v/>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Eliminar descarga sin conexión</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Supprimer le téléchargement hors connexion</t>
+        </is>
       </c>
     </row>
     <row r="318">
@@ -7008,13 +7060,15 @@
           <t>Save offline</t>
         </is>
       </c>
-      <c r="C325">
-        <f>_xlfn.TRANSLATE($B325,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D325">
-        <f>_xlfn.TRANSLATE($B325,$B$2,D$2)</f>
-        <v/>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Guardar sin conexión</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Enregistrer hors connexion</t>
+        </is>
       </c>
     </row>
     <row r="326">
@@ -8628,13 +8682,15 @@
           <t>Delete media file</t>
         </is>
       </c>
-      <c r="C406">
-        <f>_xlfn.TRANSLATE($B406,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D406">
-        <f>_xlfn.TRANSLATE($B406,$B$2,D$2)</f>
-        <v/>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Eliminar archivo multimedia</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Supprimer le fichier multimédia</t>
+        </is>
       </c>
     </row>
     <row r="407">
@@ -13842,13 +13898,15 @@
           <t>Discover</t>
         </is>
       </c>
-      <c r="C647">
-        <f>_xlfn.TRANSLATE($B647,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D647">
-        <f>_xlfn.TRANSLATE($B647,$B$2,D$2)</f>
-        <v/>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Descubre</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Découvrez</t>
+        </is>
       </c>
     </row>
     <row r="648">
@@ -13902,13 +13960,15 @@
           <t>No similar songs found</t>
         </is>
       </c>
-      <c r="C650">
-        <f>_xlfn.TRANSLATE($B650,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D650">
-        <f>_xlfn.TRANSLATE($B650,$B$2,D$2)</f>
-        <v/>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>No se han encontrado canciones similares</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Aucun morceau similaire trouvé</t>
+        </is>
       </c>
     </row>
     <row r="651">
@@ -13922,13 +13982,15 @@
           <t>Similar to</t>
         </is>
       </c>
-      <c r="C651">
-        <f>_xlfn.TRANSLATE($B651,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D651">
-        <f>_xlfn.TRANSLATE($B651,$B$2,D$2)</f>
-        <v/>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Similar a</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Similaire à</t>
+        </is>
       </c>
     </row>
     <row r="652">
@@ -13942,13 +14004,15 @@
           <t>Playlist created</t>
         </is>
       </c>
-      <c r="C652">
-        <f>_xlfn.TRANSLATE($B652,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D652">
-        <f>_xlfn.TRANSLATE($B652,$B$2,D$2)</f>
-        <v/>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Playlist creada</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Playlist créée</t>
+        </is>
       </c>
     </row>
     <row r="653">
@@ -13962,13 +14026,15 @@
           <t>Similar to this song</t>
         </is>
       </c>
-      <c r="C653">
-        <f>_xlfn.TRANSLATE($B653,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D653">
-        <f>_xlfn.TRANSLATE($B653,$B$2,D$2)</f>
-        <v/>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Canciones similares</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Morceaux similaires</t>
+        </is>
       </c>
     </row>
     <row r="654">
@@ -14042,19 +14108,21 @@
           <t>External suggestions are unavailable right now. Showing local picks.</t>
         </is>
       </c>
-      <c r="C657">
-        <f>_xlfn.TRANSLATE($B657,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D657">
-        <f>_xlfn.TRANSLATE($B657,$B$2,D$2)</f>
-        <v/>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Las sugerencias externas no están disponibles. Mostramos recomendaciones locales.</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Les suggestions externes sont indisponibles. Voici des recommandations locales.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(KB-28): validate header contrast and bound progressive blur cost
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -4930,13 +4930,15 @@
           <t>Log in</t>
         </is>
       </c>
-      <c r="C220">
-        <f>_xlfn.TRANSLATE(B220,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D220">
-        <f>_xlfn.TRANSLATE(B220,$B$2,D$2)</f>
-        <v/>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Se connecter</t>
+        </is>
       </c>
     </row>
     <row r="221">

</xml_diff>

<commit_message>
fix(KB-33): balance Friends columns and bound initial social feeds
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D668"/>
+  <dimension ref="A1:D670"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5694,13 +5694,15 @@
           <t>No results</t>
         </is>
       </c>
-      <c r="C258">
-        <f>_xlfn.TRANSLATE(B258,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D258">
-        <f>_xlfn.TRANSLATE(B258,$B$2,D$2)</f>
-        <v/>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Sin resultados</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Aucun résultat</t>
+        </is>
       </c>
     </row>
     <row r="259">
@@ -14360,6 +14362,50 @@
       <c r="D668" t="inlineStr">
         <is>
           <t>Récentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHOW_ALL_SHARES</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Show all {count} shared tracks</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Ver los {count} compartidos</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Voir les {count} partages</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHOW_ALL_RECENT</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Show all {count} listens</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Ver las {count} escuchas</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Voir les {count} écoutes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(KB-36): keep reward previews proportional to Friends content
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D838"/>
+  <dimension ref="A1:D839"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18105,6 +18105,28 @@
         </is>
       </c>
     </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>FRIENDS_SESSION_MILESTONES</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Session milestones</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Hitos de la sesión</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Étapes de la session</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Refactor notification and vocabulary managers; update audio bounds response handling
- Updated notificationManager to import EWebSocketMessage and rockIt.
- Removed unused friendsVocabulary import and simplified vocabulary proxy logic in vocabularyManager.
- Cleaned up silence.py by removing unnecessary line breaks and improving readability.
- Adjusted audioBoundsResponse generation command in comments for clarity.
- Added getAudioBounds method to BaseHttp for fetching audio bounds.
- Modified Vocabulary interface to include new keys and removed deprecated ones.
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D865"/>
+  <dimension ref="A1:D868"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -646,43 +646,45 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADD_TO_LIBRARY</t>
+          <t>FRIENDS_SHOW_ALL_SHARES</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Add to library</t>
+          <t>Show all {count} shared tracks</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Añadir a la biblioteca</t>
+          <t>Ver los {count} compartidos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ajouter à la bibliothèque</t>
+          <t>Voir les {count} partages</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ADD_TO_LIKED</t>
+          <t>FRIENDS_SHOW_ALL_RECENT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Add to liked</t>
-        </is>
-      </c>
-      <c r="C11">
-        <f>_xlfn.TRANSLATE(B11,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D11">
-        <f>_xlfn.TRANSLATE(B11,$B$2,D$2)</f>
-        <v/>
+          <t>Show all {count} listens</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ver las {count} escuchas</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Voir les {count} écoutes</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -18061,97 +18063,32 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>FRIENDS_SHOW_ALL_SHARES</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Show all {count} shared tracks</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Ver los {count} compartidos</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Voir les {count} partages</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>FRIENDS_SHOW_ALL_RECENT</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Show all {count} listens</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Ver las {count} escuchas</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Voir les {count} écoutes</t>
+    <row r="837"/>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>NOTIFICATION_EVENT_APPLICATION_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Application messages</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Mensajes de la aplicación</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Application messages</t>
         </is>
       </c>
     </row>
     <row r="839">
       <c r="A839" t="inlineStr">
         <is>
-          <t>FRIENDS_SESSION_MILESTONES</t>
-        </is>
-      </c>
-      <c r="B839" t="inlineStr">
-        <is>
-          <t>Session milestones</t>
-        </is>
-      </c>
-      <c r="C839" t="inlineStr">
-        <is>
-          <t>Hitos de la sesión</t>
-        </is>
-      </c>
-      <c r="D839" t="inlineStr">
-        <is>
-          <t>Étapes de la session</t>
-        </is>
-      </c>
-    </row>
-    <row r="838">
-      <c r="A838" t="inlineStr">
-        <is>
-          <t>NOTIFICATION_EVENT_APPLICATION_MESSAGE</t>
-        </is>
-      </c>
-      <c r="B838" t="inlineStr">
-        <is>
-          <t>Application messages</t>
-        </is>
-      </c>
-      <c r="C838" t="inlineStr">
-        <is>
-          <t>Mensajes de la aplicación</t>
-        </is>
-      </c>
-      <c r="D838" t="inlineStr">
-        <is>
-          <t>Application messages</t>
-        </is>
-      </c>
-    </row>
-    <row r="839">
-      <c r="A839" t="inlineStr">
-        <is>
           <t>NOTIFICATION_APPLICATION_MESSAGE</t>
         </is>
       </c>
@@ -18740,6 +18677,72 @@
       <c r="D865" t="inlineStr">
         <is>
           <t>ZIP ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>ADD_TO_LIBRARY</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Add to library</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Añadir a la biblioteca</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Ajouter à la bibliothèque</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>ADD_TO_LIKED</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Add to liked songs</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Añadir a canciones que me gustan</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Ajouter aux titres aimés</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>FRIENDS_SESSION_MILESTONES</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Session milestones</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Hitos de la sesión</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Étapes de la session</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(lyrics): preserve sources and apply reviewed recording-bound corrections
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D889" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:D889"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D912" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D912"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -435,12 +435,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D889"/>
+  <dimension ref="A1:D912"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -19211,10 +19211,516 @@
         </is>
       </c>
     </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>LYRICS_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>No lyrics available</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>No hay letra disponible</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Aucune parole disponible</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>LYRICS_LOADING</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Loading lyrics…</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Cargando letra…</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Chargement des paroles…</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>LYRICS_LOCAL_REQUIRED</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Download this recording before proposing corrections.</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Descarga esta grabación antes de proponer correcciones.</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Téléchargez cet enregistrement avant de proposer des corrections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>LYRICS_PREVIEW</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Preview lyrics with audio</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Escuchar y comprobar la letra</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Écouter et vérifier les paroles</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>LYRICS_PREVIEW_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Audio preview unavailable.</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>La previsualización de audio no está disponible.</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Aperçu audio indisponible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>LYRICS_CORRECTION_TITLE</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Propose a lyrics correction</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Proponer una corrección de letra</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Proposer une correction des paroles</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>LYRICS_APPROVED</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Correction reviewed by an admin</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Corrección revisada por un admin</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Correction examinée par un administrateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>LYRICS_PROVIDER_TIMING</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Provider timing: alignment with this recording has not been verified.</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Tiempos del proveedor: no se ha verificado su sincronía con esta grabación.</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Horodatage du fournisseur : synchronisation non vérifiée pour cet enregistrement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>LYRICS_OFFSET_LABEL</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Advance lyrics (seconds)</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Adelantar letra (segundos)</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Avancer les paroles (secondes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>LYRICS_OFFSET_HELP</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Positive values show lyrics earlier; negative values delay them. Preview only until approved.</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Los valores positivos adelantan la letra; los negativos la retrasan. Solo es una prueba hasta su aprobación.</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Les valeurs positives avancent les paroles ; les négatives les retardent. Aperçu uniquement avant approbation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>LYRICS_EDIT_LINES</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Edit text and line times</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Editar texto y tiempos por línea</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Modifier le texte et les temps des lignes</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>LYRICS_TIME</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Time in seconds, optional</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Tiempo en segundos, opcional</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Temps en secondes, facultatif</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>LYRICS_TEXT</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Lyrics line</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Línea de letra</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Ligne de paroles</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>LYRICS_REMOVE_LINE</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Remove line</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Eliminar línea</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Supprimer la ligne</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>LYRICS_ADD_LINE</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Add line</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Añadir línea</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Ajouter une ligne</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>LYRICS_REVIEW_HELP</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Check the beginning, middle and end. A changing delay needs line corrections, not a global offset.</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Comprueba el inicio, la mitad y el final. Si el desfase cambia, corrige las líneas: un offset global no basta.</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Vérifiez le début, le milieu et la fin. Un décalage variable nécessite une correction des lignes, pas un décalage global.</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>LYRICS_PROPOSAL_SENT</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Proposal sent for admin review. Originals remain unchanged.</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Propuesta enviada para revisión. Los originales se conservan.</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Proposition envoyée pour examen. Les originaux sont conservés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>LYRICS_PROPOSE</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Submit lyrics proposal</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Enviar propuesta de letra</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Envoyer la proposition de paroles</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>LYRICS_LEGACY_PROPOSAL</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>This old proposal has no source revision. Request a new proposal before applying it.</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Esta propuesta antigua no identifica la revisión original. Solicita una nueva antes de aplicarla.</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>Cette ancienne proposition ne précise pas la révision source. Demandez une nouvelle proposition avant application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>LYRICS_STALE_PROPOSAL</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Audio, lyrics or an approved correction have changed. This proposal needs to be recreated.</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Han cambiado el audio, la letra o una corrección aprobada. Hay que volver a crear esta propuesta.</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>L’audio, les paroles ou une correction approuvée ont changé. Cette proposition doit être recréée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>LYRICS_SHOW_CURRENT</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Compare with current lyrics</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Comparar con la letra actual</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>Comparer avec les paroles actuelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>LYRICS_SHOW_PROPOSED</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Preview proposed lyrics</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Previsualizar la propuesta</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>Prévisualiser la proposition</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>LYRICS_INVALID_CORRECTION</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Use valid numbers and ordered times for every line, or leave all times empty.</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Usa números válidos y tiempos ordenados en todas las líneas, o deja todos los tiempos vacíos.</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>Utilisez des nombres valides et des temps ordonnés pour chaque ligne, ou laissez tous les temps vides.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart ns1:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(library): drag songs and albums into owned playlists
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D657" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A2:D657"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D874" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D874"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -435,12 +435,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D868"/>
+  <dimension ref="A1:D874"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18746,10 +18746,142 @@
         </is>
       </c>
     </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>LIBRARY_DROP_ERROR</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Could not add the item. Please try again.</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>No se ha podido añadir. Inténtalo de nuevo.</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Impossible d’ajouter cet élément. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>LIBRARY_DROP_OWNER_ONLY</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Drop items into a playlist you own.</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Solo puedes soltar elementos en tus propias playlists.</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Déposez les éléments dans une playlist qui vous appartient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>LIBRARY_DROP_SUCCESS</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Added “{media}” to “{playlist}”.</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Se ha añadido «{media}» a «{playlist}».</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>« {media} » ajouté à « {playlist} ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>LIBRARY_DRAGGING</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Dragging {media}.</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Arrastrando {media}.</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Déplacement de {media}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>LIBRARY_DROP_TARGET</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Release to add to {playlist}.</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Suelta para añadir a {playlist}.</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Relâchez pour ajouter à {playlist}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>LIBRARY_DROP_SAVING</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Adding to playlist…</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Añadiendo a la playlist…</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Ajout à la playlist…</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(library): search individual songs inside saved collections
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D874" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:D874"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D876" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D876"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D874"/>
+  <dimension ref="A1:D876"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18878,6 +18878,50 @@
         </is>
       </c>
     </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>LIBRARY_SONG_SEARCH_HINT</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Songs in your Library, albums and playlists.</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Canciones de tu Library, álbumes y playlists.</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Titres de votre bibliothèque, albums et playlists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>LIBRARY_SONG_SEARCH_INCOMPLETE</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Could not search inside collections. Showing available results; please try again.</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>No se ha podido buscar dentro de las colecciones. Se muestran los resultados disponibles; inténtalo de nuevo.</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Impossible de rechercher dans les collections. Les résultats disponibles sont affichés ; réessayez.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(navigation): persist personal album playlist and artist pins
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D876" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:D876"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D887" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D887"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D876"/>
+  <dimension ref="A1:D887"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18922,6 +18922,248 @@
         </is>
       </c>
     </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>NAV_LABEL</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Main navigation</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Navegación principal</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Navigation principale</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>NAV_TOGGLE</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Expand or collapse navigation</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Expandir o contraer navegación</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Développer ou réduire la navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>NAV_PINNED</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Pinned</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Fijados</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>Épinglés</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>NAV_PIN</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Pin to navigation</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Fijar en navegación</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Épingler à la navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>NAV_UNPIN</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Unpin from navigation</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Desfijar de navegación</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Désépingler de la navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>NAV_UNPIN_ITEM</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Unpin {name}</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Desfijar {name}</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>Désépingler {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>NAV_PINS_LOADING</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Loading pinned items…</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Cargando fijados…</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>Chargement des éléments épinglés…</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>NAV_PINS_RETRY</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Retry loading pinned items</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Reintentar cargar fijados</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>Réessayer de charger les éléments épinglés</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>NAV_PINS_UPDATE_ERROR</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Could not update pinned items. Please try again.</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>No se han podido actualizar los fijados. Inténtalo de nuevo.</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Impossible de modifier les éléments épinglés. Réessayez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>NAV_PIN_ADDED</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Pinned to navigation.</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Fijado en navegación.</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Épinglé à la navigation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>NAV_PIN_REMOVED</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Unpinned from navigation.</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Desfijado de navegación.</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Désépinglé de la navigation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(navigation): contextual anchors and default Rockit lists for new users
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D887" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:D887"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D889" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D889"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D887"/>
+  <dimension ref="A1:D889"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6124,9 +6124,10 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C279">
-        <f>_xlfn.TRANSLATE(B279,$B$2,C$2)</f>
-        <v/>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Anclar</t>
+        </is>
       </c>
       <c r="D279">
         <f>_xlfn.TRANSLATE(B279,$B$2,D$2)</f>
@@ -6144,9 +6145,10 @@
           <t>Pinned Lists</t>
         </is>
       </c>
-      <c r="C280">
-        <f>_xlfn.TRANSLATE(B280,$B$2,C$2)</f>
-        <v/>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Listas ancladas</t>
+        </is>
       </c>
       <c r="D280">
         <f>_xlfn.TRANSLATE(B280,$B$2,D$2)</f>
@@ -7785,9 +7787,10 @@
           <t>Unpin</t>
         </is>
       </c>
-      <c r="C360">
-        <f>_xlfn.TRANSLATE(B360,$B$2,C$2)</f>
-        <v/>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Desanclar</t>
+        </is>
       </c>
       <c r="D360">
         <f>_xlfn.TRANSLATE(B360,$B$2,D$2)</f>
@@ -18979,7 +18982,7 @@
       </c>
       <c r="C879" t="inlineStr">
         <is>
-          <t>Fijados</t>
+          <t>Anclados</t>
         </is>
       </c>
       <c r="D879" t="inlineStr">
@@ -19001,7 +19004,7 @@
       </c>
       <c r="C880" t="inlineStr">
         <is>
-          <t>Fijar en navegación</t>
+          <t>Anclar en navegación</t>
         </is>
       </c>
       <c r="D880" t="inlineStr">
@@ -19023,7 +19026,7 @@
       </c>
       <c r="C881" t="inlineStr">
         <is>
-          <t>Desfijar de navegación</t>
+          <t>Desanclar de navegación</t>
         </is>
       </c>
       <c r="D881" t="inlineStr">
@@ -19045,7 +19048,7 @@
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>Desfijar {name}</t>
+          <t>Desanclar {name}</t>
         </is>
       </c>
       <c r="D882" t="inlineStr">
@@ -19067,7 +19070,7 @@
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>Cargando fijados…</t>
+          <t>Cargando anclados…</t>
         </is>
       </c>
       <c r="D883" t="inlineStr">
@@ -19089,7 +19092,7 @@
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>Reintentar cargar fijados</t>
+          <t>Reintentar cargar anclados</t>
         </is>
       </c>
       <c r="D884" t="inlineStr">
@@ -19111,7 +19114,7 @@
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>No se han podido actualizar los fijados. Inténtalo de nuevo.</t>
+          <t>No se han podido actualizar los anclados. Inténtalo de nuevo.</t>
         </is>
       </c>
       <c r="D885" t="inlineStr">
@@ -19133,7 +19136,7 @@
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>Fijado en navegación.</t>
+          <t>Anclado en navegación.</t>
         </is>
       </c>
       <c r="D886" t="inlineStr">
@@ -19155,12 +19158,56 @@
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>Desfijado de navegación.</t>
+          <t>Desanclado de navegación.</t>
         </is>
       </c>
       <c r="D887" t="inlineStr">
         <is>
           <t>Désépinglé de la navigation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>NAV_LAST_MONTH</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Last month’s mix</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Mix del mes pasado</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>Mix du mois dernier</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>NAV_YEAR_RECAP</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Year recap</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Resumen anual</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Récapitulatif annuel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ios): retain native audio and recover background track endings
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D912" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:D912"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A1:D913" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D913"/>
   <sortState ref="A3:D401">
     <sortCondition ref="A2:A401"/>
   </sortState>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D912"/>
+  <dimension ref="A1:D913"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -19717,6 +19717,28 @@
         </is>
       </c>
     </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>SETTINGS_TRANSITIONS_IOS_NATIVE</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>On iPhone and iPad, transitions are disabled to preserve background playback.</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>En iPhone y iPad, las transiciones están desactivadas para mantener la reproducción en segundo plano.</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>Sur iPhone et iPad, les transitions sont désactivées pour préserver la lecture en arrière-plan.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>